<commit_message>
Market: elektrik yükü tablosu (Excel + plan), cihaz numaraları
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XWsgQSXSw4djjBeQMbCe9D
</commit_message>
<xml_diff>
--- a/proje/market_havalandirma/ISI_KAZANCI_VE_KLIMA_SANTRALI_HESABI.xlsx
+++ b/proje/market_havalandirma/ISI_KAZANCI_VE_KLIMA_SANTRALI_HESABI.xlsx
@@ -12,34 +12,43 @@
     <sheet name="MAHALLER" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="KS HESABI" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="CİHAZ LİSTESİ" sheetId="4" state="visible" r:id="rId6"/>
-    <sheet name="KONTROL" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="ELEKTRİK YÜKLERİ" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="KONTROL" sheetId="6" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="false" name="cam_oran" vbProcedure="false">VARSAYIMLAR!$B$30</definedName>
+    <definedName function="false" hidden="false" name="cam_oran" vbProcedure="false">VARSAYIMLAR!$B$39</definedName>
+    <definedName function="false" hidden="false" name="COP" vbProcedure="false">VARSAYIMLAR!$B$28</definedName>
+    <definedName function="false" hidden="false" name="cos_du" vbProcedure="false">VARSAYIMLAR!$B$31</definedName>
+    <definedName function="false" hidden="false" name="cos_ks" vbProcedure="false">VARSAYIMLAR!$B$30</definedName>
     <definedName function="false" hidden="false" name="cp" vbProcedure="false">VARSAYIMLAR!$B$16</definedName>
     <definedName function="false" hidden="false" name="dus" vbProcedure="false">VARSAYIMLAR!$B$23</definedName>
+    <definedName function="false" hidden="false" name="EER" vbProcedure="false">VARSAYIMLAR!$B$27</definedName>
     <definedName function="false" hidden="false" name="emn" vbProcedure="false">VARSAYIMLAR!$B$22</definedName>
     <definedName function="false" hidden="false" name="eps" vbProcedure="false">VARSAYIMLAR!$B$18</definedName>
-    <definedName function="false" hidden="false" name="f_zemin" vbProcedure="false">VARSAYIMLAR!$B$28</definedName>
+    <definedName function="false" hidden="false" name="f_zemin" vbProcedure="false">VARSAYIMLAR!$B$37</definedName>
     <definedName function="false" hidden="false" name="hfg" vbProcedure="false">VARSAYIMLAR!$B$17</definedName>
-    <definedName function="false" hidden="false" name="n_siz" vbProcedure="false">VARSAYIMLAR!$B$31</definedName>
+    <definedName function="false" hidden="false" name="k_donus" vbProcedure="false">VARSAYIMLAR!$B$25</definedName>
+    <definedName function="false" hidden="false" name="k_sig" vbProcedure="false">VARSAYIMLAR!$B$32</definedName>
+    <definedName function="false" hidden="false" name="n_siz" vbProcedure="false">VARSAYIMLAR!$B$40</definedName>
     <definedName function="false" hidden="false" name="Patm" vbProcedure="false">VARSAYIMLAR!$B$12</definedName>
     <definedName function="false" hidden="false" name="P_fan" vbProcedure="false">VARSAYIMLAR!$B$19</definedName>
+    <definedName function="false" hidden="false" name="P_oto" vbProcedure="false">VARSAYIMLAR!$B$26</definedName>
     <definedName function="false" hidden="false" name="q_alan" vbProcedure="false">VARSAYIMLAR!$B$21</definedName>
     <definedName function="false" hidden="false" name="q_kisi" vbProcedure="false">VARSAYIMLAR!$B$20</definedName>
     <definedName function="false" hidden="false" name="rho" vbProcedure="false">VARSAYIMLAR!$B$15</definedName>
     <definedName function="false" hidden="false" name="RH_kis" vbProcedure="false">VARSAYIMLAR!$B$10</definedName>
     <definedName function="false" hidden="false" name="RH_yaz" vbProcedure="false">VARSAYIMLAR!$B$8</definedName>
-    <definedName function="false" hidden="false" name="TIP_TABLO" vbProcedure="false">VARSAYIMLAR!$A$35:$D$37</definedName>
+    <definedName function="false" hidden="false" name="TIP_TABLO" vbProcedure="false">VARSAYIMLAR!$A$44:$D$46</definedName>
     <definedName function="false" hidden="false" name="Ti_kis" vbProcedure="false">VARSAYIMLAR!$B$11</definedName>
     <definedName function="false" hidden="false" name="Ti_yaz" vbProcedure="false">VARSAYIMLAR!$B$7</definedName>
     <definedName function="false" hidden="false" name="To_kis" vbProcedure="false">VARSAYIMLAR!$B$9</definedName>
     <definedName function="false" hidden="false" name="To_yaz" vbProcedure="false">VARSAYIMLAR!$B$5</definedName>
     <definedName function="false" hidden="false" name="Twb_yaz" vbProcedure="false">VARSAYIMLAR!$B$6</definedName>
-    <definedName function="false" hidden="false" name="U_cam" vbProcedure="false">VARSAYIMLAR!$B$29</definedName>
-    <definedName function="false" hidden="false" name="U_cati" vbProcedure="false">VARSAYIMLAR!$B$25</definedName>
-    <definedName function="false" hidden="false" name="U_duvar" vbProcedure="false">VARSAYIMLAR!$B$26</definedName>
-    <definedName function="false" hidden="false" name="U_zemin" vbProcedure="false">VARSAYIMLAR!$B$27</definedName>
+    <definedName function="false" hidden="false" name="U_cam" vbProcedure="false">VARSAYIMLAR!$B$38</definedName>
+    <definedName function="false" hidden="false" name="U_cati" vbProcedure="false">VARSAYIMLAR!$B$34</definedName>
+    <definedName function="false" hidden="false" name="U_duvar" vbProcedure="false">VARSAYIMLAR!$B$35</definedName>
+    <definedName function="false" hidden="false" name="U_v" vbProcedure="false">VARSAYIMLAR!$B$29</definedName>
+    <definedName function="false" hidden="false" name="U_zemin" vbProcedure="false">VARSAYIMLAR!$B$36</definedName>
     <definedName function="false" hidden="false" name="V_ks" vbProcedure="false">VARSAYIMLAR!$B$14</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
@@ -52,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="385" uniqueCount="250">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="460" uniqueCount="291">
   <si>
     <t xml:space="preserve">ISI KAZANCI (m³ YÖNTEMİ) VE KLİMA SANTRALİ HESABI — VARSAYIMLAR</t>
   </si>
@@ -186,6 +195,54 @@
     <t xml:space="preserve">ısı pompası −3 °C dış havada nominal ısıtmanın ~%80’i</t>
   </si>
   <si>
+    <t xml:space="preserve">ELEKTRİK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dönüş/egzoz fanı gücü / üfleme fanı gücü</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dönüş tarafı dış statik basınç daha düşük</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Santral otomasyon + damper motorları</t>
+  </si>
+  <si>
+    <t xml:space="preserve">santral başına (varsayım)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dış ünite soğutma verimi EER (35 °C dış hava)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hava kaynaklı DX ısı pompası (varsayım, üretici değeriyle değiştir)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dış ünite ısıtma verimi COP (−3 °C dış hava)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">varsayım, üretici değeriyle değiştir</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Besleme gerilimi (3 faz)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">V</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3~ 50 Hz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Güç faktörü — EC fanlı santral</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Güç faktörü — inverter dış ünite</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sigorta seçim katsayısı</t>
+  </si>
+  <si>
+    <t xml:space="preserve">In ≥ 1,25 × I</t>
+  </si>
+  <si>
     <t xml:space="preserve">KABUK (ISI KAYBI)</t>
   </si>
   <si>
@@ -745,6 +802,81 @@
   </si>
   <si>
     <t xml:space="preserve">Dış ünite ölçüleri ve adet üretici seçimine göre kesinleşecektir; ölçüler yerleşim için yaklaşık verilmiştir. Ünite ölçüleri çizimdeki kesit ve yerleşim paftasıyla aynıdır.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ISITMA-SOĞUTMA VE HAVALANDIRMA CİHAZLARI ELEKTRİK YÜKÜ TABLOSU</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cihaz numaraları planda cihaz yanındaki daire içindeki numaralarla aynıdır. Dış ünite gücü soğutma ve ısıtma çekişinin büyüğüdür. Kablo kesiti ve pano seçimi elektrik projesinde yapılacaktır.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CİHAZ KODU</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GÜÇ BİLEŞENLERİ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SOĞUTMA ÇEKİŞİ (kW)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ISITMA ÇEKİŞİ (kW)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ELEKTRİK GÜCÜ (kW)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GERİLİM (V)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cos φ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AKIM (A)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SİGORTA (A)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">üfleme EC fanı + dönüş EC fanı + otomasyon</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DÜ-1.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DX DIŞ ÜNİTE (ISI POMPASI)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">kompresör + kondenser fanları</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DÜ-1.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DÜ-2.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DÜ-2.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DÜ-3.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DÜ-3.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DÜ-4.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DÜ-4.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOPLAM KURULU GÜÇ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EŞ ZAMANLI ÇEKİŞ (soğutma modu, eş zamanlılık 1,0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EŞ ZAMANLI ÇEKİŞ (ısıtma modu)</t>
   </si>
   <si>
     <t xml:space="preserve">KONTROL — MARKET BİRİM ISI KAZANCININ BİLEŞENLERLE DOĞRULANMASI (m² başına)</t>
@@ -808,7 +940,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="10">
+  <numFmts count="11">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="#,##0.##"/>
     <numFmt numFmtId="166" formatCode="0.000"/>
@@ -819,6 +951,7 @@
     <numFmt numFmtId="171" formatCode="0.00000"/>
     <numFmt numFmtId="172" formatCode="0.0%"/>
     <numFmt numFmtId="173" formatCode="0%"/>
+    <numFmt numFmtId="174" formatCode="0"/>
   </numFmts>
   <fonts count="11">
     <font>
@@ -966,7 +1099,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="38">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1099,11 +1232,23 @@
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="174" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="174" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1359,7 +1504,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:F39"/>
+  <dimension ref="A1:F48"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44"/>
@@ -1648,66 +1793,66 @@
         <v>45</v>
       </c>
       <c r="B25" s="7" t="n">
-        <v>0.2</v>
+        <v>0.8</v>
       </c>
       <c r="C25" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D25" s="6" t="s">
         <v>46</v>
-      </c>
-      <c r="D25" s="6" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="B26" s="7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="D26" s="6" t="s">
         <v>48</v>
-      </c>
-      <c r="B26" s="7" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="C26" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="D26" s="6" t="s">
-        <v>49</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="B27" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D27" s="6" t="s">
         <v>50</v>
-      </c>
-      <c r="B27" s="7" t="n">
-        <v>0.35</v>
-      </c>
-      <c r="C27" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="D27" s="6" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B28" s="7" t="n">
-        <v>0.5</v>
+        <v>2.6</v>
       </c>
       <c r="C28" s="4" t="s">
         <v>11</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>400</v>
+      </c>
+      <c r="C29" s="4" t="s">
         <v>54</v>
-      </c>
-      <c r="B29" s="7" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="C29" s="4" t="s">
-        <v>46</v>
       </c>
       <c r="D29" s="6" t="s">
         <v>55</v>
@@ -1718,120 +1863,236 @@
         <v>56</v>
       </c>
       <c r="B30" s="7" t="n">
-        <v>0.5</v>
+        <v>0.95</v>
       </c>
       <c r="C30" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="D30" s="6" t="s">
-        <v>57</v>
-      </c>
+      <c r="D30" s="6"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="B31" s="7" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D31" s="6"/>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="B31" s="7" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="C31" s="4" t="s">
+      <c r="B32" s="7" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="C32" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D32" s="6" t="s">
         <v>59</v>
-      </c>
-      <c r="D31" s="6" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="B33" s="3"/>
+      <c r="C33" s="3"/>
+      <c r="D33" s="3"/>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="4" t="s">
         <v>61</v>
       </c>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="8" t="s">
+      <c r="B34" s="7" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C34" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="B34" s="8" t="s">
+      <c r="D34" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="C34" s="8" t="s">
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="D34" s="8" t="s">
+      <c r="B35" s="7" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="D35" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="E34" s="8" t="s">
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="F34" s="8" t="s">
+      <c r="B36" s="7" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="C36" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="D36" s="6" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="9" t="s">
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="B35" s="10" t="n">
+      <c r="B37" s="7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C37" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D37" s="6" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="B38" s="7" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="C38" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="D38" s="6" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="B39" s="7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C39" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D39" s="6" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="B40" s="7" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="C40" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="D40" s="6" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="3" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="B43" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="C43" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="D43" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="E43" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="F43" s="8" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="B44" s="10" t="n">
         <v>12</v>
       </c>
-      <c r="C35" s="11" t="n">
+      <c r="C44" s="11" t="n">
         <v>0.8</v>
       </c>
-      <c r="D35" s="11" t="n">
+      <c r="D44" s="11" t="n">
         <v>0.15</v>
       </c>
-      <c r="E35" s="12" t="n">
-        <f aca="false">B35*6</f>
+      <c r="E44" s="12" t="n">
+        <f aca="false">B44*6</f>
         <v>72</v>
       </c>
-      <c r="F35" s="13" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="B36" s="10" t="n">
+      <c r="F44" s="13" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="9" t="s">
+        <v>86</v>
+      </c>
+      <c r="B45" s="10" t="n">
         <v>15</v>
       </c>
-      <c r="C36" s="11" t="n">
+      <c r="C45" s="11" t="n">
         <v>0.85</v>
       </c>
-      <c r="D36" s="11" t="n">
+      <c r="D45" s="11" t="n">
         <v>0.05</v>
       </c>
-      <c r="E36" s="12" t="n">
-        <f aca="false">B36*4.5</f>
+      <c r="E45" s="12" t="n">
+        <f aca="false">B45*4.5</f>
         <v>67.5</v>
       </c>
-      <c r="F36" s="13" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="9" t="s">
-        <v>72</v>
-      </c>
-      <c r="B37" s="10" t="n">
+      <c r="F45" s="13" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="B46" s="10" t="n">
         <v>20</v>
       </c>
-      <c r="C37" s="11" t="n">
+      <c r="C46" s="11" t="n">
         <v>0.85</v>
       </c>
-      <c r="D37" s="11" t="n">
+      <c r="D46" s="11" t="n">
         <v>0.15</v>
       </c>
-      <c r="E37" s="12" t="n">
-        <f aca="false">B37*4.5</f>
+      <c r="E46" s="12" t="n">
+        <f aca="false">B46*4.5</f>
         <v>90</v>
       </c>
-      <c r="F37" s="13" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="2" t="s">
-        <v>74</v>
+      <c r="F46" s="13" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="2" t="s">
+        <v>90</v>
       </c>
     </row>
   </sheetData>
@@ -1860,103 +2121,103 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>75</v>
+        <v>91</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>76</v>
+        <v>92</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
-        <v>77</v>
+        <v>93</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>78</v>
+        <v>94</v>
       </c>
       <c r="C4" s="14" t="s">
+        <v>95</v>
+      </c>
+      <c r="D4" s="14" t="s">
+        <v>96</v>
+      </c>
+      <c r="E4" s="14" t="s">
+        <v>97</v>
+      </c>
+      <c r="F4" s="14" t="s">
+        <v>98</v>
+      </c>
+      <c r="G4" s="14" t="s">
+        <v>99</v>
+      </c>
+      <c r="H4" s="14" t="s">
         <v>79</v>
       </c>
-      <c r="D4" s="14" t="s">
-        <v>80</v>
-      </c>
-      <c r="E4" s="14" t="s">
-        <v>81</v>
-      </c>
-      <c r="F4" s="14" t="s">
-        <v>82</v>
-      </c>
-      <c r="G4" s="14" t="s">
-        <v>83</v>
-      </c>
-      <c r="H4" s="14" t="s">
-        <v>63</v>
-      </c>
       <c r="I4" s="14" t="s">
-        <v>84</v>
+        <v>100</v>
       </c>
       <c r="J4" s="14" t="s">
-        <v>85</v>
+        <v>101</v>
       </c>
       <c r="K4" s="14" t="s">
-        <v>86</v>
+        <v>102</v>
       </c>
       <c r="L4" s="14" t="s">
-        <v>87</v>
+        <v>103</v>
       </c>
       <c r="M4" s="14" t="s">
-        <v>88</v>
+        <v>104</v>
       </c>
       <c r="N4" s="14" t="s">
-        <v>89</v>
+        <v>105</v>
       </c>
       <c r="O4" s="14" t="s">
-        <v>90</v>
+        <v>106</v>
       </c>
       <c r="P4" s="14" t="s">
-        <v>91</v>
+        <v>107</v>
       </c>
       <c r="Q4" s="14" t="s">
-        <v>92</v>
+        <v>108</v>
       </c>
       <c r="R4" s="14" t="s">
-        <v>93</v>
+        <v>109</v>
       </c>
       <c r="S4" s="14" t="s">
-        <v>94</v>
+        <v>110</v>
       </c>
       <c r="T4" s="14" t="s">
-        <v>95</v>
+        <v>111</v>
       </c>
       <c r="U4" s="14" t="s">
-        <v>96</v>
+        <v>112</v>
       </c>
       <c r="V4" s="14" t="s">
-        <v>97</v>
+        <v>113</v>
       </c>
       <c r="W4" s="14" t="s">
-        <v>98</v>
+        <v>114</v>
       </c>
       <c r="X4" s="14" t="s">
-        <v>99</v>
+        <v>115</v>
       </c>
       <c r="Y4" s="14" t="s">
-        <v>100</v>
+        <v>116</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="15" t="s">
-        <v>101</v>
+        <v>117</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>102</v>
+        <v>118</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>103</v>
+        <v>119</v>
       </c>
       <c r="D5" s="16" t="s">
-        <v>68</v>
+        <v>84</v>
       </c>
       <c r="E5" s="17" t="n">
         <v>1750.3</v>
@@ -2040,16 +2301,16 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="15" t="s">
-        <v>101</v>
+        <v>117</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>104</v>
+        <v>120</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>70</v>
+        <v>86</v>
       </c>
       <c r="D6" s="16" t="s">
-        <v>70</v>
+        <v>86</v>
       </c>
       <c r="E6" s="17" t="n">
         <v>371.3</v>
@@ -2133,16 +2394,16 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="15" t="s">
-        <v>101</v>
+        <v>117</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>105</v>
+        <v>121</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>72</v>
+        <v>88</v>
       </c>
       <c r="D7" s="16" t="s">
-        <v>72</v>
+        <v>88</v>
       </c>
       <c r="E7" s="17" t="n">
         <v>265.2</v>
@@ -2226,16 +2487,16 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="15" t="s">
-        <v>106</v>
+        <v>122</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>102</v>
+        <v>118</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>103</v>
+        <v>119</v>
       </c>
       <c r="D8" s="16" t="s">
-        <v>68</v>
+        <v>84</v>
       </c>
       <c r="E8" s="17" t="n">
         <v>1617.3</v>
@@ -2319,16 +2580,16 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="15" t="s">
-        <v>106</v>
+        <v>122</v>
       </c>
       <c r="B9" s="16" t="s">
-        <v>104</v>
+        <v>120</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>70</v>
+        <v>86</v>
       </c>
       <c r="D9" s="16" t="s">
-        <v>70</v>
+        <v>86</v>
       </c>
       <c r="E9" s="17" t="n">
         <v>330.2</v>
@@ -2412,16 +2673,16 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="15" t="s">
-        <v>106</v>
+        <v>122</v>
       </c>
       <c r="B10" s="16" t="s">
-        <v>107</v>
+        <v>123</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>72</v>
+        <v>88</v>
       </c>
       <c r="D10" s="16" t="s">
-        <v>72</v>
+        <v>88</v>
       </c>
       <c r="E10" s="17" t="n">
         <v>264.9</v>
@@ -2505,16 +2766,16 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="15" t="s">
-        <v>108</v>
+        <v>124</v>
       </c>
       <c r="B11" s="16" t="s">
-        <v>102</v>
+        <v>118</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>103</v>
+        <v>119</v>
       </c>
       <c r="D11" s="16" t="s">
-        <v>68</v>
+        <v>84</v>
       </c>
       <c r="E11" s="17" t="n">
         <v>1741.7</v>
@@ -2598,16 +2859,16 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="15" t="s">
-        <v>108</v>
+        <v>124</v>
       </c>
       <c r="B12" s="16" t="s">
-        <v>104</v>
+        <v>120</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>70</v>
+        <v>86</v>
       </c>
       <c r="D12" s="16" t="s">
-        <v>70</v>
+        <v>86</v>
       </c>
       <c r="E12" s="17" t="n">
         <v>237.7</v>
@@ -2691,16 +2952,16 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="15" t="s">
-        <v>108</v>
+        <v>124</v>
       </c>
       <c r="B13" s="16" t="s">
-        <v>109</v>
+        <v>125</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>72</v>
+        <v>88</v>
       </c>
       <c r="D13" s="16" t="s">
-        <v>72</v>
+        <v>88</v>
       </c>
       <c r="E13" s="17" t="n">
         <v>220.7</v>
@@ -2784,16 +3045,16 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="15" t="s">
-        <v>110</v>
+        <v>126</v>
       </c>
       <c r="B14" s="16" t="s">
-        <v>102</v>
+        <v>118</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>103</v>
+        <v>119</v>
       </c>
       <c r="D14" s="16" t="s">
-        <v>68</v>
+        <v>84</v>
       </c>
       <c r="E14" s="17" t="n">
         <v>1885.3</v>
@@ -2877,16 +3138,16 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="15" t="s">
-        <v>110</v>
+        <v>126</v>
       </c>
       <c r="B15" s="16" t="s">
-        <v>104</v>
+        <v>120</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>70</v>
+        <v>86</v>
       </c>
       <c r="D15" s="16" t="s">
-        <v>70</v>
+        <v>86</v>
       </c>
       <c r="E15" s="17" t="n">
         <v>211.5</v>
@@ -2970,16 +3231,16 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="15" t="s">
-        <v>110</v>
+        <v>126</v>
       </c>
       <c r="B16" s="16" t="s">
-        <v>111</v>
+        <v>127</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>72</v>
+        <v>88</v>
       </c>
       <c r="D16" s="16" t="s">
-        <v>72</v>
+        <v>88</v>
       </c>
       <c r="E16" s="17" t="n">
         <v>265.9</v>
@@ -3063,7 +3324,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="23" t="s">
-        <v>112</v>
+        <v>128</v>
       </c>
       <c r="B17" s="24"/>
       <c r="C17" s="24"/>
@@ -3134,7 +3395,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="26" t="s">
-        <v>113</v>
+        <v>129</v>
       </c>
     </row>
   </sheetData>
@@ -3164,40 +3425,40 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>114</v>
+        <v>130</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>115</v>
+        <v>131</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>116</v>
+        <v>132</v>
       </c>
       <c r="B4" s="8" t="s">
+        <v>133</v>
+      </c>
+      <c r="C4" s="8" t="s">
         <v>117</v>
       </c>
-      <c r="C4" s="8" t="s">
-        <v>101</v>
-      </c>
       <c r="D4" s="8" t="s">
-        <v>106</v>
+        <v>122</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>108</v>
+        <v>124</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>110</v>
+        <v>126</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>118</v>
+        <v>134</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>119</v>
+        <v>135</v>
       </c>
       <c r="B5" s="27"/>
       <c r="C5" s="27"/>
@@ -3208,10 +3469,10 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>120</v>
+        <v>136</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>121</v>
+        <v>137</v>
       </c>
       <c r="C6" s="19" t="n">
         <f aca="false">SUMIF(MAHALLER!$A$5:$A$16,C$4,MAHALLER!$G$5:$G$16)</f>
@@ -3230,15 +3491,15 @@
         <v>13460.1</v>
       </c>
       <c r="G6" s="13" t="s">
-        <v>122</v>
+        <v>138</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>123</v>
+        <v>139</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>124</v>
+        <v>140</v>
       </c>
       <c r="C7" s="19" t="n">
         <f aca="false">SUMIF(MAHALLER!$A$5:$A$16,C$4,MAHALLER!$E$5:$E$16)</f>
@@ -3260,7 +3521,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>125</v>
+        <v>141</v>
       </c>
       <c r="B8" s="16" t="s">
         <v>32</v>
@@ -3282,12 +3543,12 @@
         <v>173.94885</v>
       </c>
       <c r="G8" s="13" t="s">
-        <v>126</v>
+        <v>142</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>127</v>
+        <v>143</v>
       </c>
       <c r="B9" s="16" t="s">
         <v>32</v>
@@ -3312,7 +3573,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>128</v>
+        <v>144</v>
       </c>
       <c r="B10" s="16" t="s">
         <v>32</v>
@@ -3337,7 +3598,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>129</v>
+        <v>145</v>
       </c>
       <c r="B11" s="16" t="s">
         <v>32</v>
@@ -3359,12 +3620,12 @@
         <v>56.51795313</v>
       </c>
       <c r="G11" s="13" t="s">
-        <v>130</v>
+        <v>146</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>131</v>
+        <v>147</v>
       </c>
       <c r="B12" s="16" t="s">
         <v>21</v>
@@ -3386,12 +3647,12 @@
         <v>14370.804</v>
       </c>
       <c r="G12" s="13" t="s">
-        <v>132</v>
+        <v>148</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>133</v>
+        <v>149</v>
       </c>
       <c r="B13" s="27"/>
       <c r="C13" s="27"/>
@@ -3402,10 +3663,10 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>134</v>
+        <v>150</v>
       </c>
       <c r="B14" s="16" t="s">
-        <v>135</v>
+        <v>151</v>
       </c>
       <c r="C14" s="19" t="n">
         <f aca="false">SUMIF(MAHALLER!$A$5:$A$16,C$4,MAHALLER!$L$5:$L$16)</f>
@@ -3424,12 +3685,12 @@
         <v>334</v>
       </c>
       <c r="G14" s="13" t="s">
-        <v>136</v>
+        <v>152</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>137</v>
+        <v>153</v>
       </c>
       <c r="B15" s="16" t="s">
         <v>21</v>
@@ -3451,15 +3712,15 @@
         <v>40000</v>
       </c>
       <c r="G15" s="13" t="s">
-        <v>138</v>
+        <v>154</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>139</v>
+        <v>155</v>
       </c>
       <c r="B16" s="16" t="s">
-        <v>140</v>
+        <v>156</v>
       </c>
       <c r="C16" s="28" t="n">
         <f aca="false">C15*rho/3600</f>
@@ -3481,7 +3742,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>141</v>
+        <v>157</v>
       </c>
       <c r="B17" s="16" t="s">
         <v>21</v>
@@ -3503,12 +3764,12 @@
         <v>14500</v>
       </c>
       <c r="G17" s="13" t="s">
-        <v>142</v>
+        <v>158</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>143</v>
+        <v>159</v>
       </c>
       <c r="B18" s="16" t="s">
         <v>11</v>
@@ -3530,12 +3791,12 @@
         <v>0.3625</v>
       </c>
       <c r="G18" s="13" t="s">
-        <v>144</v>
+        <v>160</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>145</v>
+        <v>161</v>
       </c>
       <c r="B19" s="16" t="s">
         <v>21</v>
@@ -3557,15 +3818,15 @@
         <v>14500</v>
       </c>
       <c r="G19" s="13" t="s">
-        <v>146</v>
+        <v>162</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>147</v>
+        <v>163</v>
       </c>
       <c r="B20" s="16" t="s">
-        <v>148</v>
+        <v>164</v>
       </c>
       <c r="C20" s="12" t="n">
         <f aca="false">P_fan/(C16*cp)</f>
@@ -3584,12 +3845,12 @@
         <v>1.26739562624254</v>
       </c>
       <c r="G20" s="13" t="s">
-        <v>149</v>
+        <v>165</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="3" t="s">
-        <v>150</v>
+        <v>166</v>
       </c>
       <c r="B21" s="27"/>
       <c r="C21" s="27"/>
@@ -3600,10 +3861,10 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
-        <v>151</v>
+        <v>167</v>
       </c>
       <c r="B22" s="16" t="s">
-        <v>152</v>
+        <v>168</v>
       </c>
       <c r="C22" s="29" t="n">
         <f aca="false">((2501-2.326*Twb_yaz)*(0.622*0.61094*EXP(17.625*Twb_yaz/(Twb_yaz+243.04))/(Patm-0.61094*EXP(17.625*Twb_yaz/(Twb_yaz+243.04))))-1.006*(To_yaz-Twb_yaz))/(2501+1.86*To_yaz-4.186*Twb_yaz)</f>
@@ -3622,15 +3883,15 @@
         <v>0.0157955602769311</v>
       </c>
       <c r="G22" s="13" t="s">
-        <v>153</v>
+        <v>169</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="4" t="s">
-        <v>154</v>
+        <v>170</v>
       </c>
       <c r="B23" s="16" t="s">
-        <v>152</v>
+        <v>168</v>
       </c>
       <c r="C23" s="29" t="n">
         <f aca="false">0.622*RH_yaz*0.61094*EXP(17.625*Ti_yaz/(Ti_yaz+243.04))/(Patm-RH_yaz*0.61094*EXP(17.625*Ti_yaz/(Ti_yaz+243.04)))</f>
@@ -3652,7 +3913,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="s">
-        <v>155</v>
+        <v>171</v>
       </c>
       <c r="B24" s="16" t="s">
         <v>4</v>
@@ -3674,12 +3935,12 @@
         <v>28.25</v>
       </c>
       <c r="G24" s="13" t="s">
-        <v>156</v>
+        <v>172</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
-        <v>157</v>
+        <v>173</v>
       </c>
       <c r="B25" s="16" t="s">
         <v>4</v>
@@ -3704,10 +3965,10 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
-        <v>158</v>
+        <v>174</v>
       </c>
       <c r="B26" s="16" t="s">
-        <v>152</v>
+        <v>168</v>
       </c>
       <c r="C26" s="29" t="n">
         <f aca="false">C18*C22+(1-C18)*C23</f>
@@ -3729,7 +3990,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
-        <v>159</v>
+        <v>175</v>
       </c>
       <c r="B27" s="16" t="s">
         <v>28</v>
@@ -3754,7 +4015,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
-        <v>160</v>
+        <v>176</v>
       </c>
       <c r="B28" s="16" t="s">
         <v>4</v>
@@ -3776,15 +4037,15 @@
         <v>15.4828944458251</v>
       </c>
       <c r="G28" s="13" t="s">
-        <v>161</v>
+        <v>177</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="s">
-        <v>162</v>
+        <v>178</v>
       </c>
       <c r="B29" s="16" t="s">
-        <v>152</v>
+        <v>168</v>
       </c>
       <c r="C29" s="29" t="n">
         <f aca="false">C23-C10/(C16*hfg)</f>
@@ -3803,12 +4064,12 @@
         <v>0.00948571793804389</v>
       </c>
       <c r="G29" s="13" t="s">
-        <v>163</v>
+        <v>179</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="4" t="s">
-        <v>164</v>
+        <v>180</v>
       </c>
       <c r="B30" s="16" t="s">
         <v>4</v>
@@ -3830,15 +4091,15 @@
         <v>14.2154988195825</v>
       </c>
       <c r="G30" s="13" t="s">
-        <v>165</v>
+        <v>181</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="4" t="s">
-        <v>166</v>
+        <v>182</v>
       </c>
       <c r="B31" s="16" t="s">
-        <v>167</v>
+        <v>183</v>
       </c>
       <c r="C31" s="30" t="n">
         <f aca="false">(C29*Patm/(0.622+C29))/(0.61094*EXP(17.625*C30/(C30+243.04)))</f>
@@ -3857,12 +4118,12 @@
         <v>0.940704997074278</v>
       </c>
       <c r="G31" s="13" t="s">
-        <v>168</v>
+        <v>184</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="4" t="s">
-        <v>169</v>
+        <v>185</v>
       </c>
       <c r="B32" s="16" t="s">
         <v>28</v>
@@ -3887,7 +4148,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="4" t="s">
-        <v>170</v>
+        <v>186</v>
       </c>
       <c r="B33" s="16" t="s">
         <v>32</v>
@@ -3909,12 +4170,12 @@
         <v>271.148011210085</v>
       </c>
       <c r="G33" s="13" t="s">
-        <v>171</v>
+        <v>187</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="4" t="s">
-        <v>172</v>
+        <v>188</v>
       </c>
       <c r="B34" s="16" t="s">
         <v>32</v>
@@ -3939,7 +4200,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="4" t="s">
-        <v>173</v>
+        <v>189</v>
       </c>
       <c r="B35" s="16" t="s">
         <v>32</v>
@@ -3964,10 +4225,10 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="4" t="s">
-        <v>174</v>
+        <v>190</v>
       </c>
       <c r="B36" s="16" t="s">
-        <v>175</v>
+        <v>191</v>
       </c>
       <c r="C36" s="19" t="n">
         <f aca="false">C16*(C26-C29)*3600</f>
@@ -3986,12 +4247,12 @@
         <v>139.9624842906</v>
       </c>
       <c r="G36" s="13" t="s">
-        <v>176</v>
+        <v>192</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="23" t="s">
-        <v>177</v>
+        <v>193</v>
       </c>
       <c r="B37" s="16" t="s">
         <v>32</v>
@@ -4013,12 +4274,12 @@
         <v>300</v>
       </c>
       <c r="G37" s="13" t="s">
-        <v>178</v>
+        <v>194</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="3" t="s">
-        <v>179</v>
+        <v>195</v>
       </c>
       <c r="B38" s="27"/>
       <c r="C38" s="27"/>
@@ -4029,7 +4290,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="4" t="s">
-        <v>155</v>
+        <v>171</v>
       </c>
       <c r="B39" s="16" t="s">
         <v>4</v>
@@ -4051,12 +4312,12 @@
         <v>14.25</v>
       </c>
       <c r="G39" s="13" t="s">
-        <v>180</v>
+        <v>196</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="4" t="s">
-        <v>157</v>
+        <v>173</v>
       </c>
       <c r="B40" s="16" t="s">
         <v>4</v>
@@ -4081,7 +4342,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="4" t="s">
-        <v>160</v>
+        <v>176</v>
       </c>
       <c r="B41" s="16" t="s">
         <v>4</v>
@@ -4103,12 +4364,12 @@
         <v>24.2135650941849</v>
       </c>
       <c r="G41" s="13" t="s">
-        <v>181</v>
+        <v>197</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="4" t="s">
-        <v>164</v>
+        <v>180</v>
       </c>
       <c r="B42" s="16" t="s">
         <v>4</v>
@@ -4130,12 +4391,12 @@
         <v>22.9461694679423</v>
       </c>
       <c r="G42" s="13" t="s">
-        <v>165</v>
+        <v>181</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="4" t="s">
-        <v>182</v>
+        <v>198</v>
       </c>
       <c r="B43" s="16" t="s">
         <v>32</v>
@@ -4157,12 +4418,12 @@
         <v>67.4763697966667</v>
       </c>
       <c r="G43" s="13" t="s">
-        <v>183</v>
+        <v>199</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="4" t="s">
-        <v>184</v>
+        <v>200</v>
       </c>
       <c r="B44" s="16" t="s">
         <v>32</v>
@@ -4184,12 +4445,12 @@
         <v>123.584619796667</v>
       </c>
       <c r="G44" s="13" t="s">
-        <v>185</v>
+        <v>201</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="23" t="s">
-        <v>186</v>
+        <v>202</v>
       </c>
       <c r="B45" s="16" t="s">
         <v>32</v>
@@ -4211,12 +4472,12 @@
         <v>140</v>
       </c>
       <c r="G45" s="13" t="s">
-        <v>187</v>
+        <v>203</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="3" t="s">
-        <v>188</v>
+        <v>204</v>
       </c>
       <c r="B46" s="27"/>
       <c r="C46" s="27"/>
@@ -4227,7 +4488,7 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="4" t="s">
-        <v>189</v>
+        <v>205</v>
       </c>
       <c r="B47" s="16" t="s">
         <v>32</v>
@@ -4252,7 +4513,7 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="4" t="s">
-        <v>190</v>
+        <v>206</v>
       </c>
       <c r="B48" s="16" t="s">
         <v>32</v>
@@ -4277,7 +4538,7 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="4" t="s">
-        <v>191</v>
+        <v>207</v>
       </c>
       <c r="B49" s="16" t="s">
         <v>32</v>
@@ -4299,15 +4560,15 @@
         <v>175</v>
       </c>
       <c r="G49" s="13" t="s">
-        <v>192</v>
+        <v>208</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="4" t="s">
-        <v>193</v>
+        <v>209</v>
       </c>
       <c r="B50" s="16" t="s">
-        <v>194</v>
+        <v>210</v>
       </c>
       <c r="C50" s="19" t="n">
         <f aca="false">2</f>
@@ -4326,12 +4587,12 @@
         <v>2</v>
       </c>
       <c r="G50" s="13" t="s">
-        <v>195</v>
+        <v>211</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="4" t="s">
-        <v>196</v>
+        <v>212</v>
       </c>
       <c r="B51" s="16" t="s">
         <v>32</v>
@@ -4356,7 +4617,7 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="4" t="s">
-        <v>197</v>
+        <v>213</v>
       </c>
       <c r="B52" s="16" t="s">
         <v>32</v>
@@ -4381,7 +4642,7 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="3" t="s">
-        <v>198</v>
+        <v>214</v>
       </c>
       <c r="B53" s="27"/>
       <c r="C53" s="27"/>
@@ -4392,7 +4653,7 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="4" t="s">
-        <v>199</v>
+        <v>215</v>
       </c>
       <c r="B54" s="16" t="s">
         <v>32</v>
@@ -4414,12 +4675,12 @@
         <v>200</v>
       </c>
       <c r="G54" s="13" t="s">
-        <v>200</v>
+        <v>216</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="4" t="s">
-        <v>201</v>
+        <v>217</v>
       </c>
       <c r="B55" s="16" t="s">
         <v>11</v>
@@ -4441,12 +4702,12 @@
         <v>1.5</v>
       </c>
       <c r="G55" s="13" t="s">
-        <v>202</v>
+        <v>218</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="23" t="s">
-        <v>203</v>
+        <v>219</v>
       </c>
       <c r="B56" s="16" t="s">
         <v>32</v>
@@ -4458,7 +4719,7 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="23" t="s">
-        <v>204</v>
+        <v>220</v>
       </c>
       <c r="B57" s="16" t="s">
         <v>32</v>
@@ -4470,7 +4731,7 @@
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="23" t="s">
-        <v>205</v>
+        <v>221</v>
       </c>
       <c r="B58" s="16" t="s">
         <v>32</v>
@@ -4508,44 +4769,44 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>206</v>
+        <v>222</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
-        <v>207</v>
+        <v>223</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>208</v>
+        <v>224</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>209</v>
+        <v>225</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>101</v>
+        <v>117</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>106</v>
+        <v>122</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>108</v>
+        <v>124</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>110</v>
+        <v>126</v>
       </c>
       <c r="H3" s="8" t="s">
-        <v>117</v>
+        <v>133</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="15" t="s">
-        <v>77</v>
+        <v>93</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>210</v>
+        <v>226</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>211</v>
+        <v>227</v>
       </c>
       <c r="D4" s="19" t="n">
         <f aca="false">'KS HESABI'!C15</f>
@@ -4570,10 +4831,10 @@
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="15"/>
       <c r="B5" s="9" t="s">
-        <v>212</v>
+        <v>228</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>213</v>
+        <v>229</v>
       </c>
       <c r="D5" s="19" t="n">
         <f aca="false">'KS HESABI'!C17</f>
@@ -4625,7 +4886,7 @@
       <c r="A7" s="15"/>
       <c r="B7" s="4"/>
       <c r="C7" s="4" t="s">
-        <v>214</v>
+        <v>230</v>
       </c>
       <c r="D7" s="22" t="n">
         <f aca="false">'KS HESABI'!C37</f>
@@ -4651,7 +4912,7 @@
       <c r="A8" s="15"/>
       <c r="B8" s="4"/>
       <c r="C8" s="4" t="s">
-        <v>215</v>
+        <v>231</v>
       </c>
       <c r="D8" s="22" t="n">
         <f aca="false">'KS HESABI'!C45</f>
@@ -4677,7 +4938,7 @@
       <c r="A9" s="15"/>
       <c r="B9" s="4"/>
       <c r="C9" s="4" t="s">
-        <v>174</v>
+        <v>190</v>
       </c>
       <c r="D9" s="19" t="n">
         <f aca="false">'KS HESABI'!C36</f>
@@ -4696,14 +4957,14 @@
         <v>139.9624842906</v>
       </c>
       <c r="H9" s="16" t="s">
-        <v>175</v>
+        <v>191</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="15"/>
       <c r="B10" s="4"/>
       <c r="C10" s="4" t="s">
-        <v>216</v>
+        <v>232</v>
       </c>
       <c r="D10" s="22" t="n">
         <f aca="false">P_fan</f>
@@ -4729,22 +4990,22 @@
       <c r="A11" s="15"/>
       <c r="B11" s="4"/>
       <c r="C11" s="4" t="s">
-        <v>217</v>
+        <v>233</v>
       </c>
       <c r="D11" s="22" t="n">
-        <f aca="false">ROUND(P_fan*0.8,1)</f>
+        <f aca="false">ROUND(P_fan*k_donus,1)</f>
         <v>13.6</v>
       </c>
       <c r="E11" s="22" t="n">
-        <f aca="false">ROUND(P_fan*0.8,1)</f>
+        <f aca="false">ROUND(P_fan*k_donus,1)</f>
         <v>13.6</v>
       </c>
       <c r="F11" s="22" t="n">
-        <f aca="false">ROUND(P_fan*0.8,1)</f>
+        <f aca="false">ROUND(P_fan*k_donus,1)</f>
         <v>13.6</v>
       </c>
       <c r="G11" s="22" t="n">
-        <f aca="false">ROUND(P_fan*0.8,1)</f>
+        <f aca="false">ROUND(P_fan*k_donus,1)</f>
         <v>13.6</v>
       </c>
       <c r="H11" s="16" t="s">
@@ -4755,19 +5016,19 @@
       <c r="A12" s="15"/>
       <c r="B12" s="4"/>
       <c r="C12" s="4" t="s">
-        <v>218</v>
+        <v>234</v>
       </c>
       <c r="D12" s="19" t="s">
-        <v>219</v>
+        <v>235</v>
       </c>
       <c r="E12" s="19" t="s">
-        <v>219</v>
+        <v>235</v>
       </c>
       <c r="F12" s="19" t="s">
-        <v>219</v>
+        <v>235</v>
       </c>
       <c r="G12" s="19" t="s">
-        <v>219</v>
+        <v>235</v>
       </c>
       <c r="H12" s="16"/>
     </row>
@@ -4775,33 +5036,33 @@
       <c r="A13" s="15"/>
       <c r="B13" s="4"/>
       <c r="C13" s="4" t="s">
-        <v>220</v>
+        <v>236</v>
       </c>
       <c r="D13" s="19" t="s">
-        <v>221</v>
+        <v>237</v>
       </c>
       <c r="E13" s="19" t="s">
-        <v>221</v>
+        <v>237</v>
       </c>
       <c r="F13" s="19" t="s">
-        <v>221</v>
+        <v>237</v>
       </c>
       <c r="G13" s="19" t="s">
-        <v>221</v>
+        <v>237</v>
       </c>
       <c r="H13" s="16" t="s">
-        <v>222</v>
+        <v>238</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="15" t="s">
-        <v>223</v>
+        <v>239</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>224</v>
+        <v>240</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>225</v>
+        <v>241</v>
       </c>
       <c r="D14" s="19" t="n">
         <f aca="false">'KS HESABI'!C50</f>
@@ -4820,14 +5081,14 @@
         <v>2</v>
       </c>
       <c r="H14" s="16" t="s">
-        <v>194</v>
+        <v>210</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="15"/>
       <c r="B15" s="4"/>
       <c r="C15" s="4" t="s">
-        <v>226</v>
+        <v>242</v>
       </c>
       <c r="D15" s="22" t="n">
         <f aca="false">'KS HESABI'!C51</f>
@@ -4853,7 +5114,7 @@
       <c r="A16" s="15"/>
       <c r="B16" s="4"/>
       <c r="C16" s="4" t="s">
-        <v>227</v>
+        <v>243</v>
       </c>
       <c r="D16" s="22" t="n">
         <f aca="false">'KS HESABI'!C52</f>
@@ -4879,27 +5140,27 @@
       <c r="A17" s="15"/>
       <c r="B17" s="4"/>
       <c r="C17" s="4" t="s">
-        <v>228</v>
+        <v>244</v>
       </c>
       <c r="D17" s="19" t="s">
-        <v>229</v>
+        <v>245</v>
       </c>
       <c r="E17" s="19" t="s">
-        <v>229</v>
+        <v>245</v>
       </c>
       <c r="F17" s="19" t="s">
-        <v>229</v>
+        <v>245</v>
       </c>
       <c r="G17" s="19" t="s">
-        <v>229</v>
+        <v>245</v>
       </c>
       <c r="H17" s="16" t="s">
-        <v>222</v>
+        <v>238</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>230</v>
+        <v>246</v>
       </c>
     </row>
   </sheetData>
@@ -4918,6 +5179,630 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
+  <dimension ref="A1:K19"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="5" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="11"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="14" t="s">
+        <v>223</v>
+      </c>
+      <c r="B4" s="14" t="s">
+        <v>249</v>
+      </c>
+      <c r="C4" s="14" t="s">
+        <v>224</v>
+      </c>
+      <c r="D4" s="14" t="s">
+        <v>250</v>
+      </c>
+      <c r="E4" s="14" t="s">
+        <v>251</v>
+      </c>
+      <c r="F4" s="14" t="s">
+        <v>252</v>
+      </c>
+      <c r="G4" s="14" t="s">
+        <v>253</v>
+      </c>
+      <c r="H4" s="14" t="s">
+        <v>254</v>
+      </c>
+      <c r="I4" s="14" t="s">
+        <v>255</v>
+      </c>
+      <c r="J4" s="14" t="s">
+        <v>256</v>
+      </c>
+      <c r="K4" s="14" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="15" t="s">
+        <v>117</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>226</v>
+      </c>
+      <c r="D5" s="13" t="s">
+        <v>258</v>
+      </c>
+      <c r="E5" s="12" t="n">
+        <f aca="false">P_fan*(1+k_donus)+P_oto</f>
+        <v>31.1</v>
+      </c>
+      <c r="F5" s="12" t="n">
+        <f aca="false">E5</f>
+        <v>31.1</v>
+      </c>
+      <c r="G5" s="33" t="n">
+        <f aca="false">ROUND(MAX(E5,F5),1)</f>
+        <v>31.1</v>
+      </c>
+      <c r="H5" s="34" t="n">
+        <f aca="false">U_v</f>
+        <v>400</v>
+      </c>
+      <c r="I5" s="28" t="n">
+        <f aca="false">cos_ks</f>
+        <v>0.95</v>
+      </c>
+      <c r="J5" s="12" t="n">
+        <f aca="false">G5*1000/(SQRT(3)*H5*I5)</f>
+        <v>47.2515615047299</v>
+      </c>
+      <c r="K5" s="35" t="n">
+        <f aca="false">INDEX({6,10,16,20,25,32,40,50,63,80,100,125,160,200,250},MATCH(TRUE(),INDEX({6,10,16,20,25,32,40,50,63,80,100,125,160,200,250}&gt;=J5*k_sig,0),0))</f>
+        <v>63</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="15" t="s">
+        <v>259</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>260</v>
+      </c>
+      <c r="D6" s="13" t="s">
+        <v>261</v>
+      </c>
+      <c r="E6" s="12" t="n">
+        <f aca="false">'KS HESABI'!C51/EER</f>
+        <v>50</v>
+      </c>
+      <c r="F6" s="12" t="n">
+        <f aca="false">'KS HESABI'!C52*dus/COP</f>
+        <v>26.1538461538462</v>
+      </c>
+      <c r="G6" s="33" t="n">
+        <f aca="false">ROUND(MAX(E6,F6),1)</f>
+        <v>50</v>
+      </c>
+      <c r="H6" s="34" t="n">
+        <f aca="false">U_v</f>
+        <v>400</v>
+      </c>
+      <c r="I6" s="28" t="n">
+        <f aca="false">cos_du</f>
+        <v>0.92</v>
+      </c>
+      <c r="J6" s="12" t="n">
+        <f aca="false">G6*1000/(SQRT(3)*H6*I6)</f>
+        <v>78.4443300529383</v>
+      </c>
+      <c r="K6" s="35" t="n">
+        <f aca="false">INDEX({6,10,16,20,25,32,40,50,63,80,100,125,160,200,250},MATCH(TRUE(),INDEX({6,10,16,20,25,32,40,50,63,80,100,125,160,200,250}&gt;=J6*k_sig,0),0))</f>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="15" t="s">
+        <v>262</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>260</v>
+      </c>
+      <c r="D7" s="13" t="s">
+        <v>261</v>
+      </c>
+      <c r="E7" s="12" t="n">
+        <f aca="false">'KS HESABI'!C51/EER</f>
+        <v>50</v>
+      </c>
+      <c r="F7" s="12" t="n">
+        <f aca="false">'KS HESABI'!C52*dus/COP</f>
+        <v>26.1538461538462</v>
+      </c>
+      <c r="G7" s="33" t="n">
+        <f aca="false">ROUND(MAX(E7,F7),1)</f>
+        <v>50</v>
+      </c>
+      <c r="H7" s="34" t="n">
+        <f aca="false">U_v</f>
+        <v>400</v>
+      </c>
+      <c r="I7" s="28" t="n">
+        <f aca="false">cos_du</f>
+        <v>0.92</v>
+      </c>
+      <c r="J7" s="12" t="n">
+        <f aca="false">G7*1000/(SQRT(3)*H7*I7)</f>
+        <v>78.4443300529383</v>
+      </c>
+      <c r="K7" s="35" t="n">
+        <f aca="false">INDEX({6,10,16,20,25,32,40,50,63,80,100,125,160,200,250},MATCH(TRUE(),INDEX({6,10,16,20,25,32,40,50,63,80,100,125,160,200,250}&gt;=J7*k_sig,0),0))</f>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="15" t="s">
+        <v>122</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>226</v>
+      </c>
+      <c r="D8" s="13" t="s">
+        <v>258</v>
+      </c>
+      <c r="E8" s="12" t="n">
+        <f aca="false">P_fan*(1+k_donus)+P_oto</f>
+        <v>31.1</v>
+      </c>
+      <c r="F8" s="12" t="n">
+        <f aca="false">E8</f>
+        <v>31.1</v>
+      </c>
+      <c r="G8" s="33" t="n">
+        <f aca="false">ROUND(MAX(E8,F8),1)</f>
+        <v>31.1</v>
+      </c>
+      <c r="H8" s="34" t="n">
+        <f aca="false">U_v</f>
+        <v>400</v>
+      </c>
+      <c r="I8" s="28" t="n">
+        <f aca="false">cos_ks</f>
+        <v>0.95</v>
+      </c>
+      <c r="J8" s="12" t="n">
+        <f aca="false">G8*1000/(SQRT(3)*H8*I8)</f>
+        <v>47.2515615047299</v>
+      </c>
+      <c r="K8" s="35" t="n">
+        <f aca="false">INDEX({6,10,16,20,25,32,40,50,63,80,100,125,160,200,250},MATCH(TRUE(),INDEX({6,10,16,20,25,32,40,50,63,80,100,125,160,200,250}&gt;=J8*k_sig,0),0))</f>
+        <v>63</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="15" t="s">
+        <v>263</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>260</v>
+      </c>
+      <c r="D9" s="13" t="s">
+        <v>261</v>
+      </c>
+      <c r="E9" s="12" t="n">
+        <f aca="false">'KS HESABI'!D51/EER</f>
+        <v>46.6666666666667</v>
+      </c>
+      <c r="F9" s="12" t="n">
+        <f aca="false">'KS HESABI'!D52*dus/COP</f>
+        <v>26.1538461538462</v>
+      </c>
+      <c r="G9" s="33" t="n">
+        <f aca="false">ROUND(MAX(E9,F9),1)</f>
+        <v>46.7</v>
+      </c>
+      <c r="H9" s="34" t="n">
+        <f aca="false">U_v</f>
+        <v>400</v>
+      </c>
+      <c r="I9" s="28" t="n">
+        <f aca="false">cos_du</f>
+        <v>0.92</v>
+      </c>
+      <c r="J9" s="12" t="n">
+        <f aca="false">G9*1000/(SQRT(3)*H9*I9)</f>
+        <v>73.2670042694444</v>
+      </c>
+      <c r="K9" s="35" t="n">
+        <f aca="false">INDEX({6,10,16,20,25,32,40,50,63,80,100,125,160,200,250},MATCH(TRUE(),INDEX({6,10,16,20,25,32,40,50,63,80,100,125,160,200,250}&gt;=J9*k_sig,0),0))</f>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="15" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="15" t="s">
+        <v>264</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>260</v>
+      </c>
+      <c r="D10" s="13" t="s">
+        <v>261</v>
+      </c>
+      <c r="E10" s="12" t="n">
+        <f aca="false">'KS HESABI'!D51/EER</f>
+        <v>46.6666666666667</v>
+      </c>
+      <c r="F10" s="12" t="n">
+        <f aca="false">'KS HESABI'!D52*dus/COP</f>
+        <v>26.1538461538462</v>
+      </c>
+      <c r="G10" s="33" t="n">
+        <f aca="false">ROUND(MAX(E10,F10),1)</f>
+        <v>46.7</v>
+      </c>
+      <c r="H10" s="34" t="n">
+        <f aca="false">U_v</f>
+        <v>400</v>
+      </c>
+      <c r="I10" s="28" t="n">
+        <f aca="false">cos_du</f>
+        <v>0.92</v>
+      </c>
+      <c r="J10" s="12" t="n">
+        <f aca="false">G10*1000/(SQRT(3)*H10*I10)</f>
+        <v>73.2670042694444</v>
+      </c>
+      <c r="K10" s="35" t="n">
+        <f aca="false">INDEX({6,10,16,20,25,32,40,50,63,80,100,125,160,200,250},MATCH(TRUE(),INDEX({6,10,16,20,25,32,40,50,63,80,100,125,160,200,250}&gt;=J10*k_sig,0),0))</f>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="15" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="15" t="s">
+        <v>124</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>226</v>
+      </c>
+      <c r="D11" s="13" t="s">
+        <v>258</v>
+      </c>
+      <c r="E11" s="12" t="n">
+        <f aca="false">P_fan*(1+k_donus)+P_oto</f>
+        <v>31.1</v>
+      </c>
+      <c r="F11" s="12" t="n">
+        <f aca="false">E11</f>
+        <v>31.1</v>
+      </c>
+      <c r="G11" s="33" t="n">
+        <f aca="false">ROUND(MAX(E11,F11),1)</f>
+        <v>31.1</v>
+      </c>
+      <c r="H11" s="34" t="n">
+        <f aca="false">U_v</f>
+        <v>400</v>
+      </c>
+      <c r="I11" s="28" t="n">
+        <f aca="false">cos_ks</f>
+        <v>0.95</v>
+      </c>
+      <c r="J11" s="12" t="n">
+        <f aca="false">G11*1000/(SQRT(3)*H11*I11)</f>
+        <v>47.2515615047299</v>
+      </c>
+      <c r="K11" s="35" t="n">
+        <f aca="false">INDEX({6,10,16,20,25,32,40,50,63,80,100,125,160,200,250},MATCH(TRUE(),INDEX({6,10,16,20,25,32,40,50,63,80,100,125,160,200,250}&gt;=J11*k_sig,0),0))</f>
+        <v>63</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="15" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="15" t="s">
+        <v>265</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>260</v>
+      </c>
+      <c r="D12" s="13" t="s">
+        <v>261</v>
+      </c>
+      <c r="E12" s="12" t="n">
+        <f aca="false">'KS HESABI'!E51/EER</f>
+        <v>46.6666666666667</v>
+      </c>
+      <c r="F12" s="12" t="n">
+        <f aca="false">'KS HESABI'!E52*dus/COP</f>
+        <v>26.1538461538462</v>
+      </c>
+      <c r="G12" s="33" t="n">
+        <f aca="false">ROUND(MAX(E12,F12),1)</f>
+        <v>46.7</v>
+      </c>
+      <c r="H12" s="34" t="n">
+        <f aca="false">U_v</f>
+        <v>400</v>
+      </c>
+      <c r="I12" s="28" t="n">
+        <f aca="false">cos_du</f>
+        <v>0.92</v>
+      </c>
+      <c r="J12" s="12" t="n">
+        <f aca="false">G12*1000/(SQRT(3)*H12*I12)</f>
+        <v>73.2670042694444</v>
+      </c>
+      <c r="K12" s="35" t="n">
+        <f aca="false">INDEX({6,10,16,20,25,32,40,50,63,80,100,125,160,200,250},MATCH(TRUE(),INDEX({6,10,16,20,25,32,40,50,63,80,100,125,160,200,250}&gt;=J12*k_sig,0),0))</f>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="15" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" s="15" t="s">
+        <v>266</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>260</v>
+      </c>
+      <c r="D13" s="13" t="s">
+        <v>261</v>
+      </c>
+      <c r="E13" s="12" t="n">
+        <f aca="false">'KS HESABI'!E51/EER</f>
+        <v>46.6666666666667</v>
+      </c>
+      <c r="F13" s="12" t="n">
+        <f aca="false">'KS HESABI'!E52*dus/COP</f>
+        <v>26.1538461538462</v>
+      </c>
+      <c r="G13" s="33" t="n">
+        <f aca="false">ROUND(MAX(E13,F13),1)</f>
+        <v>46.7</v>
+      </c>
+      <c r="H13" s="34" t="n">
+        <f aca="false">U_v</f>
+        <v>400</v>
+      </c>
+      <c r="I13" s="28" t="n">
+        <f aca="false">cos_du</f>
+        <v>0.92</v>
+      </c>
+      <c r="J13" s="12" t="n">
+        <f aca="false">G13*1000/(SQRT(3)*H13*I13)</f>
+        <v>73.2670042694444</v>
+      </c>
+      <c r="K13" s="35" t="n">
+        <f aca="false">INDEX({6,10,16,20,25,32,40,50,63,80,100,125,160,200,250},MATCH(TRUE(),INDEX({6,10,16,20,25,32,40,50,63,80,100,125,160,200,250}&gt;=J13*k_sig,0),0))</f>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="15" t="n">
+        <v>10</v>
+      </c>
+      <c r="B14" s="15" t="s">
+        <v>126</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>226</v>
+      </c>
+      <c r="D14" s="13" t="s">
+        <v>258</v>
+      </c>
+      <c r="E14" s="12" t="n">
+        <f aca="false">P_fan*(1+k_donus)+P_oto</f>
+        <v>31.1</v>
+      </c>
+      <c r="F14" s="12" t="n">
+        <f aca="false">E14</f>
+        <v>31.1</v>
+      </c>
+      <c r="G14" s="33" t="n">
+        <f aca="false">ROUND(MAX(E14,F14),1)</f>
+        <v>31.1</v>
+      </c>
+      <c r="H14" s="34" t="n">
+        <f aca="false">U_v</f>
+        <v>400</v>
+      </c>
+      <c r="I14" s="28" t="n">
+        <f aca="false">cos_ks</f>
+        <v>0.95</v>
+      </c>
+      <c r="J14" s="12" t="n">
+        <f aca="false">G14*1000/(SQRT(3)*H14*I14)</f>
+        <v>47.2515615047299</v>
+      </c>
+      <c r="K14" s="35" t="n">
+        <f aca="false">INDEX({6,10,16,20,25,32,40,50,63,80,100,125,160,200,250},MATCH(TRUE(),INDEX({6,10,16,20,25,32,40,50,63,80,100,125,160,200,250}&gt;=J14*k_sig,0),0))</f>
+        <v>63</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="15" t="n">
+        <v>11</v>
+      </c>
+      <c r="B15" s="15" t="s">
+        <v>267</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>260</v>
+      </c>
+      <c r="D15" s="13" t="s">
+        <v>261</v>
+      </c>
+      <c r="E15" s="12" t="n">
+        <f aca="false">'KS HESABI'!F51/EER</f>
+        <v>50</v>
+      </c>
+      <c r="F15" s="12" t="n">
+        <f aca="false">'KS HESABI'!F52*dus/COP</f>
+        <v>27.6923076923077</v>
+      </c>
+      <c r="G15" s="33" t="n">
+        <f aca="false">ROUND(MAX(E15,F15),1)</f>
+        <v>50</v>
+      </c>
+      <c r="H15" s="34" t="n">
+        <f aca="false">U_v</f>
+        <v>400</v>
+      </c>
+      <c r="I15" s="28" t="n">
+        <f aca="false">cos_du</f>
+        <v>0.92</v>
+      </c>
+      <c r="J15" s="12" t="n">
+        <f aca="false">G15*1000/(SQRT(3)*H15*I15)</f>
+        <v>78.4443300529383</v>
+      </c>
+      <c r="K15" s="35" t="n">
+        <f aca="false">INDEX({6,10,16,20,25,32,40,50,63,80,100,125,160,200,250},MATCH(TRUE(),INDEX({6,10,16,20,25,32,40,50,63,80,100,125,160,200,250}&gt;=J15*k_sig,0),0))</f>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="15" t="n">
+        <v>12</v>
+      </c>
+      <c r="B16" s="15" t="s">
+        <v>268</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>260</v>
+      </c>
+      <c r="D16" s="13" t="s">
+        <v>261</v>
+      </c>
+      <c r="E16" s="12" t="n">
+        <f aca="false">'KS HESABI'!F51/EER</f>
+        <v>50</v>
+      </c>
+      <c r="F16" s="12" t="n">
+        <f aca="false">'KS HESABI'!F52*dus/COP</f>
+        <v>27.6923076923077</v>
+      </c>
+      <c r="G16" s="33" t="n">
+        <f aca="false">ROUND(MAX(E16,F16),1)</f>
+        <v>50</v>
+      </c>
+      <c r="H16" s="34" t="n">
+        <f aca="false">U_v</f>
+        <v>400</v>
+      </c>
+      <c r="I16" s="28" t="n">
+        <f aca="false">cos_du</f>
+        <v>0.92</v>
+      </c>
+      <c r="J16" s="12" t="n">
+        <f aca="false">G16*1000/(SQRT(3)*H16*I16)</f>
+        <v>78.4443300529383</v>
+      </c>
+      <c r="K16" s="35" t="n">
+        <f aca="false">INDEX({6,10,16,20,25,32,40,50,63,80,100,125,160,200,250},MATCH(TRUE(),INDEX({6,10,16,20,25,32,40,50,63,80,100,125,160,200,250}&gt;=J16*k_sig,0),0))</f>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="24"/>
+      <c r="B17" s="24"/>
+      <c r="C17" s="23" t="s">
+        <v>269</v>
+      </c>
+      <c r="D17" s="24"/>
+      <c r="E17" s="31" t="n">
+        <f aca="false">SUM(E5:E16)</f>
+        <v>511.066666666667</v>
+      </c>
+      <c r="F17" s="31" t="n">
+        <f aca="false">SUM(F5:F16)</f>
+        <v>336.707692307692</v>
+      </c>
+      <c r="G17" s="31" t="n">
+        <f aca="false">SUM(G5:G16)</f>
+        <v>511.2</v>
+      </c>
+      <c r="H17" s="24"/>
+      <c r="I17" s="24"/>
+      <c r="J17" s="31" t="n">
+        <f aca="false">SUM(J5:J16)</f>
+        <v>795.85158330845</v>
+      </c>
+      <c r="K17" s="24"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C18" s="9" t="s">
+        <v>270</v>
+      </c>
+      <c r="G18" s="36" t="n">
+        <f aca="false">E17</f>
+        <v>511.066666666667</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C19" s="9" t="s">
+        <v>271</v>
+      </c>
+      <c r="G19" s="36" t="n">
+        <f aca="false">F17</f>
+        <v>336.707692307692</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="true"/>
+  </sheetPr>
   <dimension ref="A1:E11"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
@@ -4928,125 +5813,125 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>231</v>
+        <v>272</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
-        <v>232</v>
+        <v>273</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>233</v>
+        <v>274</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>117</v>
+        <v>133</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>234</v>
+        <v>275</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>235</v>
+        <v>276</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>236</v>
-      </c>
-      <c r="B4" s="33" t="n">
+        <v>277</v>
+      </c>
+      <c r="B4" s="37" t="n">
         <f aca="false">VLOOKUP("MARKET",TIP_TABLO,4,FALSE())</f>
         <v>0.15</v>
       </c>
       <c r="C4" s="16" t="s">
-        <v>237</v>
+        <v>278</v>
       </c>
       <c r="D4" s="12" t="n">
         <f aca="false">B4*130</f>
         <v>19.5</v>
       </c>
       <c r="E4" s="13" t="s">
-        <v>238</v>
+        <v>279</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>239</v>
+        <v>280</v>
       </c>
       <c r="B5" s="11" t="n">
         <v>12</v>
       </c>
       <c r="C5" s="16" t="s">
-        <v>234</v>
+        <v>275</v>
       </c>
       <c r="D5" s="12" t="n">
         <f aca="false">B5</f>
         <v>12</v>
       </c>
       <c r="E5" s="13" t="s">
-        <v>240</v>
+        <v>281</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>241</v>
+        <v>282</v>
       </c>
       <c r="B6" s="11" t="n">
         <v>10</v>
       </c>
       <c r="C6" s="16" t="s">
-        <v>234</v>
+        <v>275</v>
       </c>
       <c r="D6" s="12" t="n">
         <f aca="false">B6</f>
         <v>10</v>
       </c>
       <c r="E6" s="13" t="s">
-        <v>57</v>
+        <v>73</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>242</v>
-      </c>
-      <c r="B7" s="33" t="n">
+        <v>283</v>
+      </c>
+      <c r="B7" s="37" t="n">
         <f aca="false">U_cati</f>
         <v>0.2</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>46</v>
+        <v>62</v>
       </c>
       <c r="D7" s="12" t="n">
         <f aca="false">B7*25</f>
         <v>5</v>
       </c>
       <c r="E7" s="13" t="s">
-        <v>243</v>
+        <v>284</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>244</v>
+        <v>285</v>
       </c>
       <c r="B8" s="11" t="n">
         <v>8</v>
       </c>
       <c r="C8" s="16" t="s">
-        <v>234</v>
+        <v>275</v>
       </c>
       <c r="D8" s="12" t="n">
         <f aca="false">B8</f>
         <v>8</v>
       </c>
       <c r="E8" s="13" t="s">
-        <v>57</v>
+        <v>73</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="9" t="s">
-        <v>245</v>
+        <v>286</v>
       </c>
       <c r="B9" s="4"/>
       <c r="C9" s="16"/>
-      <c r="D9" s="34" t="n">
+      <c r="D9" s="33" t="n">
         <f aca="false">SUM(D4:D8)</f>
         <v>54.5</v>
       </c>
@@ -5054,21 +5939,21 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>246</v>
+        <v>287</v>
       </c>
       <c r="B10" s="4"/>
       <c r="C10" s="16"/>
       <c r="D10" s="12" t="n">
-        <f aca="false">VARSAYIMLAR!E35</f>
+        <f aca="false">VARSAYIMLAR!E44</f>
         <v>72</v>
       </c>
       <c r="E10" s="13" t="s">
-        <v>247</v>
+        <v>288</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>248</v>
+        <v>289</v>
       </c>
       <c r="B11" s="4"/>
       <c r="C11" s="16"/>
@@ -5077,7 +5962,7 @@
         <v>1.32110091743119</v>
       </c>
       <c r="E11" s="13" t="s">
-        <v>249</v>
+        <v>290</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Market: santralde 2 fan motoru (üfleme + emiş), elektrik tablosu adet/birim güç düzeltmesi, araştırılmış birim güçler
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XWsgQSXSw4djjBeQMbCe9D
</commit_message>
<xml_diff>
--- a/proje/market_havalandirma/ISI_KAZANCI_VE_KLIMA_SANTRALI_HESABI.xlsx
+++ b/proje/market_havalandirma/ISI_KAZANCI_VE_KLIMA_SANTRALI_HESABI.xlsx
@@ -89,7 +89,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="569" uniqueCount="384">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="588" uniqueCount="402">
   <si>
     <t xml:space="preserve">ISI KAZANCI (m³ YÖNTEMİ) VE KLİMA SANTRALİ HESABI — VARSAYIMLAR</t>
   </si>
@@ -214,28 +214,28 @@
     <t xml:space="preserve">ısı pompası −3 °C dış havada nominal ısıtmanın ~%80’i</t>
   </si>
   <si>
-    <t xml:space="preserve">FANLAR (EC PLUG FAN DUVARI)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bölme başına fan adedi (fan duvarı)</t>
+    <t xml:space="preserve">FANLAR (SANTRALDE 2 MOTOR: 1 ÜFLEME + 1 EMİŞ/EGZOZ)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bölme başına fan / motor adedi</t>
   </si>
   <si>
     <t xml:space="preserve">adet</t>
   </si>
   <si>
-    <t xml:space="preserve">2 × 2 dizi; bir fan arızasında %75 debi sürer</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fan sistem verimi (çark + EC motor + sürücü)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EC plug fan, tasarım noktası (ihtiyatlı)</t>
+    <t xml:space="preserve">her bölmede tek fan + tek motor (üfleme ve emiş/egzoz)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fan sistem verimi (çark + motor + frekans konvertörü)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">geriye eğik kanatlı plug fan, IE4 motor, frekans konvertörlü</t>
   </si>
   <si>
     <t xml:space="preserve">Motor seçim payı</t>
   </si>
   <si>
-    <t xml:space="preserve">emilen güç × pay → bir üst standart motor gücü</t>
+    <t xml:space="preserve">motor anma gücü ≥ mil gücü × 1,10 → bir üst IEC standart motor gücü</t>
   </si>
   <si>
     <t xml:space="preserve">Kritik hat uzunluğu (santral → en uzak menfez)</t>
@@ -301,22 +301,22 @@
     <t xml:space="preserve">kW</t>
   </si>
   <si>
-    <t xml:space="preserve">adet başına, 24 V</t>
+    <t xml:space="preserve">24 V; 20 Nm sınıfı ~2 W çalışma / 4 VA boyutlandırma (Belimo LM24A 5 Nm: 1 W / 2 VA)</t>
   </si>
   <si>
     <t xml:space="preserve">Santral kontrol (DDC) panosu</t>
   </si>
   <si>
-    <t xml:space="preserve">santral başına</t>
+    <t xml:space="preserve">DDC + sensörler + 24 V trafo (varsayım)</t>
   </si>
   <si>
     <t xml:space="preserve">ELEKTRİK</t>
   </si>
   <si>
-    <t xml:space="preserve">Dış ünite soğutma verimi EER (35 °C dış hava)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">hava kaynaklı DX ısı pompası (varsayım, üretici değeriyle değiştir)</t>
+    <t xml:space="preserve">Dış ünite soğutma verimi EER (35 °C dış hava, fanlar dahil)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ısı pompalı hava soğutmalı kondenser ünitesi; Trane RAUX katalog EER 2,81 — üretici değeriyle değiştir</t>
   </si>
   <si>
     <t xml:space="preserve">Dış ünite ısıtma verimi COP (−3 °C dış hava)</t>
@@ -334,7 +334,10 @@
     <t xml:space="preserve">3~ 50 Hz</t>
   </si>
   <si>
-    <t xml:space="preserve">Güç faktörü — EC fanlı santral</t>
+    <t xml:space="preserve">Güç faktörü — frekans konvertörlü fan motorları</t>
+  </si>
+  <si>
+    <t xml:space="preserve">konvertör giriş güç faktörü</t>
   </si>
   <si>
     <t xml:space="preserve">Güç faktörü — inverter dış ünite</t>
@@ -829,16 +832,16 @@
     <t xml:space="preserve">TOPLAM ODA ISI KAZANCI (m³ yöntemi)</t>
   </si>
   <si>
-    <t xml:space="preserve">KLİMA SANTRALİ FAN HESABI — ÜFLEME VE DÖNÜŞ/EGZOZ FAN DUVARLARI (EC PLUG FAN)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fan toplam basıncı = santral iç kayıpları + dış statik basınç (kanal). Emilen güç P = V·Δp/η. Dört santral aynı fan seçimiyle donatılır (debi 40.000 m³/h). Tüm değerler ELEKTRİK gücüdür (kW).</t>
+    <t xml:space="preserve">KLİMA SANTRALİ FAN HESABI — ÜFLEME FANI VE EMİŞ / EGZOZ FANI (SANTRAL BAŞINA 2 MOTOR)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fan toplam basıncı = santral iç kayıpları + dış statik basınç (kanal). Emilen güç P = V·Δp/η. Her santralde 2 motor vardır: üfleme fanı ve emiş/egzoz fanı. Dört santral aynı seçimle donatılır. Tüm güçler ELEKTRİK gücüdür (kW).</t>
   </si>
   <si>
     <t xml:space="preserve">ÜFLEME FANI</t>
   </si>
   <si>
-    <t xml:space="preserve">DÖNÜŞ / EGZOZ FANI</t>
+    <t xml:space="preserve">EMİŞ / EGZOZ FANI</t>
   </si>
   <si>
     <t xml:space="preserve">— SANTRAL İÇ BASINÇ KAYIPLARI (Pa) —</t>
@@ -916,10 +919,13 @@
     <t xml:space="preserve">m³/h — kullanıcı projesi</t>
   </si>
   <si>
-    <t xml:space="preserve">Fan adedi (fan duvarı)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fan başına debi</t>
+    <t xml:space="preserve">Fan / motor adedi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">adet — santral başına 1 üfleme + 1 emiş</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fan debisi</t>
   </si>
   <si>
     <t xml:space="preserve">Toplam emilen elektrik gücü</t>
@@ -928,16 +934,16 @@
     <t xml:space="preserve">kW — P = V·Δp / η</t>
   </si>
   <si>
-    <t xml:space="preserve">Fan başına emilen elektrik gücü</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fan başına EC motor gücü (seçim)</t>
+    <t xml:space="preserve">Fan mil gücü (motor başına)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Motor anma gücü (seçim)</t>
   </si>
   <si>
     <t xml:space="preserve">kW — bir üst standart güç</t>
   </si>
   <si>
-    <t xml:space="preserve">Kurulu elektrik gücü (fan duvarı)</t>
+    <t xml:space="preserve">Kurulu elektrik gücü</t>
   </si>
   <si>
     <t xml:space="preserve">kW — elektrik yükü tablosuna</t>
@@ -994,28 +1000,28 @@
     <t xml:space="preserve">DX ısıtma bataryası ISIL kapasitesi</t>
   </si>
   <si>
-    <t xml:space="preserve">Üfleme fan duvarı: adet × debi</t>
+    <t xml:space="preserve">Üfleme fanı (plug fan, 1 adet) debisi</t>
   </si>
   <si>
     <t xml:space="preserve">Üfleme fanı toplam basınç / dış statik basınç</t>
   </si>
   <si>
-    <t xml:space="preserve">Üfleme fanı EC motor (fan başına)</t>
+    <t xml:space="preserve">Üfleme fanı motoru (IE4, frekans konvertörlü)</t>
   </si>
   <si>
     <t xml:space="preserve">kW elektrik</t>
   </si>
   <si>
-    <t xml:space="preserve">Dönüş/egzoz fan duvarı: adet × debi</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dönüş fanı toplam basınç / dış statik basınç</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dönüş fanı EC motor (fan başına)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Özgül fan gücü SFP (üfleme / dönüş)</t>
+    <t xml:space="preserve">Emiş / egzoz fanı (plug fan, 1 adet) debisi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Emiş fanı toplam basınç / dış statik basınç</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Emiş / egzoz fanı motoru (IE4, frekans konvertörlü)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Özgül fan gücü SFP (üfleme / emiş)</t>
   </si>
   <si>
     <t xml:space="preserve">Filtre (taze hava / dönüş / üfleme)</t>
@@ -1060,7 +1066,7 @@
     <t xml:space="preserve">ISITMA-SOĞUTMA VE HAVALANDIRMA CİHAZLARI ELEKTRİK YÜKÜ TABLOSU</t>
   </si>
   <si>
-    <t xml:space="preserve">Bu tabloda YALNIZ ELEKTRİK GÜÇLERİ vardır; ısıtma/soğutma (ısıl) kapasiteleri bu tabloda yer almaz. Numaralar planda cihaz yanındaki daire içindeki numaralardır; alt satırlar (1.1, 1.2 …) cihazın içindeki elektrik tüketicileridir. İletken kesiti ve pano seçimi elektrik projesinde yapılacaktır.</t>
+    <t xml:space="preserve">Bu tabloda YALNIZ ELEKTRİK GÜÇLERİ vardır; ısıtma/soğutma (ısıl) kapasiteleri bu tabloda yer almaz. Numaralar planda cihaz yanındaki daire içindeki numaralardır; alt satırlar (1.1, 1.2 …) cihazın içindeki elektrik tüketicileridir (2 fan motoru, damper motorları, kontrol panosu). İletken kesiti ve pano seçimi elektrik projesinde yapılacaktır.</t>
   </si>
   <si>
     <t xml:space="preserve">CİHAZ KODU</t>
@@ -1096,24 +1102,36 @@
     <t xml:space="preserve">1.1</t>
   </si>
   <si>
-    <t xml:space="preserve">Üfleme fanı — EC plug fan (fan duvarı; akım/sigorta fan başına)</t>
+    <t xml:space="preserve">KS-1/ÜF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Üfleme fanı motoru — plug fan, IE4, frekans konvertörlü</t>
   </si>
   <si>
     <t xml:space="preserve">1.2</t>
   </si>
   <si>
-    <t xml:space="preserve">Dönüş/egzoz fanı — EC plug fan (fan duvarı; akım/sigorta fan başına)</t>
+    <t xml:space="preserve">KS-1/EF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Emiş / egzoz fanı motoru — plug fan, IE4, frekans konvertörlü</t>
   </si>
   <si>
     <t xml:space="preserve">1.3</t>
   </si>
   <si>
+    <t xml:space="preserve">KS-1/DM</t>
+  </si>
+  <si>
     <t xml:space="preserve">Damper motorları — taze hava, egzoz, karışım, by-pass (230/24 V trafo, panodan)</t>
   </si>
   <si>
     <t xml:space="preserve">1.4</t>
   </si>
   <si>
+    <t xml:space="preserve">KS-1/DDC</t>
+  </si>
+  <si>
     <t xml:space="preserve">Santral kontrol (DDC) panosu (230 V)</t>
   </si>
   <si>
@@ -1129,15 +1147,27 @@
     <t xml:space="preserve">4.1</t>
   </si>
   <si>
+    <t xml:space="preserve">KS-2/ÜF</t>
+  </si>
+  <si>
     <t xml:space="preserve">4.2</t>
   </si>
   <si>
+    <t xml:space="preserve">KS-2/EF</t>
+  </si>
+  <si>
     <t xml:space="preserve">4.3</t>
   </si>
   <si>
+    <t xml:space="preserve">KS-2/DM</t>
+  </si>
+  <si>
     <t xml:space="preserve">4.4</t>
   </si>
   <si>
+    <t xml:space="preserve">KS-2/DDC</t>
+  </si>
+  <si>
     <t xml:space="preserve">DÜ-2.1</t>
   </si>
   <si>
@@ -1147,15 +1177,27 @@
     <t xml:space="preserve">7.1</t>
   </si>
   <si>
+    <t xml:space="preserve">KS-3/ÜF</t>
+  </si>
+  <si>
     <t xml:space="preserve">7.2</t>
   </si>
   <si>
+    <t xml:space="preserve">KS-3/EF</t>
+  </si>
+  <si>
     <t xml:space="preserve">7.3</t>
   </si>
   <si>
+    <t xml:space="preserve">KS-3/DM</t>
+  </si>
+  <si>
     <t xml:space="preserve">7.4</t>
   </si>
   <si>
+    <t xml:space="preserve">KS-3/DDC</t>
+  </si>
+  <si>
     <t xml:space="preserve">DÜ-3.1</t>
   </si>
   <si>
@@ -1165,13 +1207,25 @@
     <t xml:space="preserve">10.1</t>
   </si>
   <si>
+    <t xml:space="preserve">KS-4/ÜF</t>
+  </si>
+  <si>
     <t xml:space="preserve">10.2</t>
   </si>
   <si>
+    <t xml:space="preserve">KS-4/EF</t>
+  </si>
+  <si>
     <t xml:space="preserve">10.3</t>
   </si>
   <si>
+    <t xml:space="preserve">KS-4/DM</t>
+  </si>
+  <si>
     <t xml:space="preserve">10.4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">KS-4/DDC</t>
   </si>
   <si>
     <t xml:space="preserve">DÜ-4.1</t>
@@ -1407,7 +1461,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="47">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1576,7 +1630,15 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="166" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="167" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2115,7 +2177,7 @@
         <v>42</v>
       </c>
       <c r="B24" s="5" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C24" s="4" t="s">
         <v>43</v>
@@ -2129,7 +2191,7 @@
         <v>45</v>
       </c>
       <c r="B25" s="7" t="n">
-        <v>0.62</v>
+        <v>0.65</v>
       </c>
       <c r="C25" s="4" t="s">
         <v>11</v>
@@ -2143,7 +2205,7 @@
         <v>47</v>
       </c>
       <c r="B26" s="7" t="n">
-        <v>1.15</v>
+        <v>1.1</v>
       </c>
       <c r="C26" s="4" t="s">
         <v>11</v>
@@ -2277,7 +2339,7 @@
         <v>68</v>
       </c>
       <c r="B36" s="7" t="n">
-        <v>0.01</v>
+        <v>0.004</v>
       </c>
       <c r="C36" s="4" t="s">
         <v>69</v>
@@ -2291,7 +2353,7 @@
         <v>71</v>
       </c>
       <c r="B37" s="7" t="n">
-        <v>0.3</v>
+        <v>0.15</v>
       </c>
       <c r="C37" s="4" t="s">
         <v>69</v>
@@ -2313,7 +2375,7 @@
         <v>74</v>
       </c>
       <c r="B39" s="7" t="n">
-        <v>3</v>
+        <v>2.8</v>
       </c>
       <c r="C39" s="4" t="s">
         <v>11</v>
@@ -2360,11 +2422,13 @@
       <c r="C42" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="D42" s="6"/>
+      <c r="D42" s="6" t="s">
+        <v>82</v>
+      </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="4" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B43" s="7" t="n">
         <v>0.92</v>
@@ -2376,7 +2440,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="4" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B44" s="7" t="n">
         <v>1.25</v>
@@ -2385,12 +2449,12 @@
         <v>11</v>
       </c>
       <c r="D44" s="6" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="3" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B45" s="3"/>
       <c r="C45" s="3"/>
@@ -2398,49 +2462,49 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="4" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B46" s="7" t="n">
         <v>0.2</v>
       </c>
       <c r="C46" s="4" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D46" s="6" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="4" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B47" s="7" t="n">
         <v>0.25</v>
       </c>
       <c r="C47" s="4" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D47" s="6" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="4" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B48" s="7" t="n">
         <v>0.35</v>
       </c>
       <c r="C48" s="4" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D48" s="6" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="4" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B49" s="7" t="n">
         <v>0.5</v>
@@ -2449,26 +2513,26 @@
         <v>11</v>
       </c>
       <c r="D49" s="6" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="4" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B50" s="7" t="n">
         <v>1.8</v>
       </c>
       <c r="C50" s="4" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D50" s="6" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="4" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B51" s="7" t="n">
         <v>0.5</v>
@@ -2477,51 +2541,51 @@
         <v>11</v>
       </c>
       <c r="D51" s="6" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="4" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B52" s="7" t="n">
         <v>0.3</v>
       </c>
       <c r="C52" s="4" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D52" s="6" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="3" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="8" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B55" s="8" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C55" s="8" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D55" s="8" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="E55" s="8" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F55" s="8" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="9" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B56" s="10" t="n">
         <v>12</v>
@@ -2537,12 +2601,12 @@
         <v>72</v>
       </c>
       <c r="F56" s="13" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="9" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B57" s="10" t="n">
         <v>15</v>
@@ -2558,12 +2622,12 @@
         <v>67.5</v>
       </c>
       <c r="F57" s="13" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="9" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B58" s="10" t="n">
         <v>20</v>
@@ -2579,12 +2643,12 @@
         <v>90</v>
       </c>
       <c r="F58" s="13" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="2" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
   </sheetData>
@@ -2613,103 +2677,103 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="E4" s="14" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="F4" s="14" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="G4" s="14" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="H4" s="14" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="I4" s="14" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="J4" s="14" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="K4" s="14" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="L4" s="14" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="M4" s="14" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="N4" s="14" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="O4" s="14" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="P4" s="14" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="Q4" s="14" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="R4" s="14" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="S4" s="14" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="T4" s="14" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="U4" s="14" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="V4" s="14" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="W4" s="14" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="X4" s="14" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="Y4" s="14" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="15" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="D5" s="16" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E5" s="17" t="n">
         <v>1750.3</v>
@@ -2793,16 +2857,16 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="15" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D6" s="16" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="E6" s="17" t="n">
         <v>371.3</v>
@@ -2886,16 +2950,16 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="15" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D7" s="16" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="E7" s="17" t="n">
         <v>265.2</v>
@@ -2979,16 +3043,16 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="15" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="D8" s="16" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E8" s="17" t="n">
         <v>1617.3</v>
@@ -3072,16 +3136,16 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="15" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B9" s="16" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D9" s="16" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="E9" s="17" t="n">
         <v>330.2</v>
@@ -3165,16 +3229,16 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="15" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B10" s="16" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D10" s="16" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="E10" s="17" t="n">
         <v>264.9</v>
@@ -3258,16 +3322,16 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="15" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B11" s="16" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="D11" s="16" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E11" s="17" t="n">
         <v>1741.7</v>
@@ -3351,16 +3415,16 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="15" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B12" s="16" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D12" s="16" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="E12" s="17" t="n">
         <v>237.7</v>
@@ -3444,16 +3508,16 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="15" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B13" s="16" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D13" s="16" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="E13" s="17" t="n">
         <v>220.7</v>
@@ -3537,16 +3601,16 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="15" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B14" s="16" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="D14" s="16" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E14" s="17" t="n">
         <v>1885.3</v>
@@ -3630,16 +3694,16 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="15" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B15" s="16" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D15" s="16" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="E15" s="17" t="n">
         <v>211.5</v>
@@ -3723,16 +3787,16 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="15" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B16" s="16" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D16" s="16" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="E16" s="17" t="n">
         <v>265.9</v>
@@ -3816,7 +3880,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="23" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B17" s="24"/>
       <c r="C17" s="24"/>
@@ -3887,7 +3951,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="26" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
     </row>
   </sheetData>
@@ -3917,40 +3981,40 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B5" s="27"/>
       <c r="C5" s="27"/>
@@ -3961,10 +4025,10 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C6" s="19" t="n">
         <f aca="false">SUMIF(MAHALLER!$A$5:$A$16,C$4,MAHALLER!$G$5:$G$16)</f>
@@ -3983,15 +4047,15 @@
         <v>13460.1</v>
       </c>
       <c r="G6" s="13" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="C7" s="19" t="n">
         <f aca="false">SUMIF(MAHALLER!$A$5:$A$16,C$4,MAHALLER!$E$5:$E$16)</f>
@@ -4013,7 +4077,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B8" s="16" t="s">
         <v>69</v>
@@ -4035,12 +4099,12 @@
         <v>173.94885</v>
       </c>
       <c r="G8" s="13" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B9" s="16" t="s">
         <v>69</v>
@@ -4065,7 +4129,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="B10" s="16" t="s">
         <v>69</v>
@@ -4090,7 +4154,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B11" s="16" t="s">
         <v>69</v>
@@ -4112,12 +4176,12 @@
         <v>56.51795313</v>
       </c>
       <c r="G11" s="13" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B12" s="16" t="s">
         <v>21</v>
@@ -4139,12 +4203,12 @@
         <v>14370.804</v>
       </c>
       <c r="G12" s="13" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="B13" s="27"/>
       <c r="C13" s="27"/>
@@ -4155,10 +4219,10 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B14" s="16" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="C14" s="19" t="n">
         <f aca="false">SUMIF(MAHALLER!$A$5:$A$16,C$4,MAHALLER!$L$5:$L$16)</f>
@@ -4177,12 +4241,12 @@
         <v>334</v>
       </c>
       <c r="G14" s="13" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B15" s="16" t="s">
         <v>21</v>
@@ -4204,15 +4268,15 @@
         <v>40000</v>
       </c>
       <c r="G15" s="13" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B16" s="16" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="C16" s="28" t="n">
         <f aca="false">C15*rho/3600</f>
@@ -4234,7 +4298,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B17" s="16" t="s">
         <v>21</v>
@@ -4256,12 +4320,12 @@
         <v>14500</v>
       </c>
       <c r="G17" s="13" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B18" s="16" t="s">
         <v>11</v>
@@ -4283,12 +4347,12 @@
         <v>0.3625</v>
       </c>
       <c r="G18" s="13" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="B19" s="16" t="s">
         <v>21</v>
@@ -4310,39 +4374,39 @@
         <v>14500</v>
       </c>
       <c r="G19" s="13" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="B20" s="16" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="C20" s="12" t="n">
         <f aca="false">P_fan/(C16*cp)</f>
-        <v>1.25590542764916</v>
+        <v>1.19794056175766</v>
       </c>
       <c r="D20" s="12" t="n">
         <f aca="false">P_fan/(D16*cp)</f>
-        <v>1.25590542764916</v>
+        <v>1.19794056175766</v>
       </c>
       <c r="E20" s="12" t="n">
         <f aca="false">P_fan/(E16*cp)</f>
-        <v>1.25590542764916</v>
+        <v>1.19794056175766</v>
       </c>
       <c r="F20" s="12" t="n">
         <f aca="false">P_fan/(F16*cp)</f>
-        <v>1.25590542764916</v>
+        <v>1.19794056175766</v>
       </c>
       <c r="G20" s="13" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="3" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="B21" s="27"/>
       <c r="C21" s="27"/>
@@ -4353,10 +4417,10 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="B22" s="16" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="C22" s="29" t="n">
         <f aca="false">((2501-2.326*Twb_yaz)*(0.622*0.61094*EXP(17.625*Twb_yaz/(Twb_yaz+243.04))/(Patm-0.61094*EXP(17.625*Twb_yaz/(Twb_yaz+243.04))))-1.006*(To_yaz-Twb_yaz))/(2501+1.86*To_yaz-4.186*Twb_yaz)</f>
@@ -4375,15 +4439,15 @@
         <v>0.0157955602769311</v>
       </c>
       <c r="G22" s="13" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="4" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="B23" s="16" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="C23" s="29" t="n">
         <f aca="false">0.622*RH_yaz*0.61094*EXP(17.625*Ti_yaz/(Ti_yaz+243.04))/(Patm-RH_yaz*0.61094*EXP(17.625*Ti_yaz/(Ti_yaz+243.04)))</f>
@@ -4405,7 +4469,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B24" s="16" t="s">
         <v>4</v>
@@ -4427,12 +4491,12 @@
         <v>28.25</v>
       </c>
       <c r="G24" s="13" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="B25" s="16" t="s">
         <v>4</v>
@@ -4457,10 +4521,10 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="B26" s="16" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="C26" s="29" t="n">
         <f aca="false">C18*C22+(1-C18)*C23</f>
@@ -4482,7 +4546,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="B27" s="16" t="s">
         <v>28</v>
@@ -4507,7 +4571,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B28" s="16" t="s">
         <v>4</v>
@@ -4529,15 +4593,15 @@
         <v>15.4828944458251</v>
       </c>
       <c r="G28" s="13" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="B29" s="16" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="C29" s="29" t="n">
         <f aca="false">C23-C10/(C16*hfg)</f>
@@ -4556,171 +4620,171 @@
         <v>0.00948571793804389</v>
       </c>
       <c r="G29" s="13" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="4" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B30" s="16" t="s">
         <v>4</v>
       </c>
       <c r="C30" s="12" t="n">
         <f aca="false">C28-C20</f>
-        <v>14.1271648382554</v>
+        <v>14.1851297041469</v>
       </c>
       <c r="D30" s="12" t="n">
         <f aca="false">D28-D20</f>
-        <v>14.8758126389512</v>
+        <v>14.9337775048427</v>
       </c>
       <c r="E30" s="12" t="n">
         <f aca="false">E28-E20</f>
-        <v>14.9893599177783</v>
+        <v>15.0473247836698</v>
       </c>
       <c r="F30" s="12" t="n">
         <f aca="false">F28-F20</f>
-        <v>14.2269890181759</v>
+        <v>14.2849538840674</v>
       </c>
       <c r="G30" s="13" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="4" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="B31" s="16" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="C31" s="30" t="n">
         <f aca="false">(C29*Patm/(0.622+C29))/(0.61094*EXP(17.625*C30/(C30+243.04)))</f>
-        <v>0.947089044559001</v>
+        <v>0.943540757073861</v>
       </c>
       <c r="D31" s="30" t="n">
         <f aca="false">(D29*Patm/(0.622+D29))/(0.61094*EXP(17.625*D30/(D30+243.04)))</f>
-        <v>0.908941749356809</v>
+        <v>0.905556083145319</v>
       </c>
       <c r="E31" s="30" t="n">
         <f aca="false">(E29*Patm/(0.622+E29))/(0.61094*EXP(17.625*E30/(E30+243.04)))</f>
-        <v>0.901603806595213</v>
+        <v>0.898248422295962</v>
       </c>
       <c r="F31" s="30" t="n">
         <f aca="false">(F29*Patm/(0.622+F29))/(0.61094*EXP(17.625*F30/(F30+243.04)))</f>
-        <v>0.940005674318886</v>
+        <v>0.93648665186263</v>
       </c>
       <c r="G31" s="13" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="4" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="B32" s="16" t="s">
         <v>28</v>
       </c>
       <c r="C32" s="12" t="n">
         <f aca="false">cp*C30+C29*(hfg+1.86*C30)</f>
-        <v>38.2103850828375</v>
+        <v>38.2697215219289</v>
       </c>
       <c r="D32" s="12" t="n">
         <f aca="false">cp*D30+D29*(hfg+1.86*D30)</f>
-        <v>39.1538393214369</v>
+        <v>39.2131833111777</v>
       </c>
       <c r="E32" s="12" t="n">
         <f aca="false">cp*E30+E29*(hfg+1.86*E30)</f>
-        <v>39.2505150631096</v>
+        <v>39.3098582183834</v>
       </c>
       <c r="F32" s="12" t="n">
         <f aca="false">cp*F30+F29*(hfg+1.86*F30)</f>
-        <v>38.2871444765101</v>
+        <v>38.3464798309617</v>
       </c>
       <c r="G32" s="13"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="4" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="B33" s="16" t="s">
         <v>69</v>
       </c>
       <c r="C33" s="22" t="n">
         <f aca="false">C16*(C27-C32)</f>
-        <v>272.014644907571</v>
+        <v>271.223492386352</v>
       </c>
       <c r="D33" s="22" t="n">
         <f aca="false">D16*(D27-D32)</f>
-        <v>254.136807709066</v>
+        <v>253.345554512523</v>
       </c>
       <c r="E33" s="22" t="n">
         <f aca="false">E16*(E27-E32)</f>
-        <v>252.847797820097</v>
+        <v>252.05655574978</v>
       </c>
       <c r="F33" s="22" t="n">
         <f aca="false">F16*(F27-F32)</f>
-        <v>270.99118632527</v>
+        <v>270.200048265915</v>
       </c>
       <c r="G33" s="13" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="4" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B34" s="16" t="s">
         <v>69</v>
       </c>
       <c r="C34" s="22" t="n">
         <f aca="false">C16*cp*(C25-C30)</f>
-        <v>170.194545636201</v>
+        <v>169.417043568376</v>
       </c>
       <c r="D34" s="22" t="n">
         <f aca="false">D16*cp*(D25-D30)</f>
-        <v>159.398183136201</v>
+        <v>158.620681068376</v>
       </c>
       <c r="E34" s="22" t="n">
         <f aca="false">E16*cp*(E25-E30)</f>
-        <v>157.875135636201</v>
+        <v>157.097633568376</v>
       </c>
       <c r="F34" s="22" t="n">
         <f aca="false">F16*cp*(F25-F30)</f>
-        <v>168.855570636201</v>
+        <v>168.078068568376</v>
       </c>
       <c r="G34" s="13"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="4" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="B35" s="16" t="s">
         <v>69</v>
       </c>
       <c r="C35" s="22" t="n">
         <f aca="false">C33-C34</f>
-        <v>101.82009927137</v>
+        <v>101.806448817976</v>
       </c>
       <c r="D35" s="22" t="n">
         <f aca="false">D33-D34</f>
-        <v>94.7386245728657</v>
+        <v>94.7248734441472</v>
       </c>
       <c r="E35" s="22" t="n">
         <f aca="false">E33-E34</f>
-        <v>94.9726621838966</v>
+        <v>94.9589221814043</v>
       </c>
       <c r="F35" s="22" t="n">
         <f aca="false">F33-F34</f>
-        <v>102.135615689069</v>
+        <v>102.121979697539</v>
       </c>
       <c r="G35" s="13"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="4" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B36" s="16" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="C36" s="19" t="n">
         <f aca="false">C16*(C26-C29)*3600</f>
@@ -4739,12 +4803,12 @@
         <v>139.9624842906</v>
       </c>
       <c r="G36" s="13" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="23" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="B37" s="16" t="s">
         <v>69</v>
@@ -4766,12 +4830,12 @@
         <v>300</v>
       </c>
       <c r="G37" s="13" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="3" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="B38" s="27"/>
       <c r="C38" s="27"/>
@@ -4782,7 +4846,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="4" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B39" s="16" t="s">
         <v>4</v>
@@ -4804,12 +4868,12 @@
         <v>14.25</v>
       </c>
       <c r="G39" s="13" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="4" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="B40" s="16" t="s">
         <v>4</v>
@@ -4834,7 +4898,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="4" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B41" s="16" t="s">
         <v>4</v>
@@ -4856,66 +4920,66 @@
         <v>24.2135650941849</v>
       </c>
       <c r="G41" s="13" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="4" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B42" s="16" t="s">
         <v>4</v>
       </c>
       <c r="C42" s="12" t="n">
         <f aca="false">C41-C20</f>
-        <v>22.8478770827882</v>
+        <v>22.9058419486797</v>
       </c>
       <c r="D42" s="12" t="n">
         <f aca="false">D41-D20</f>
-        <v>22.5597702234443</v>
+        <v>22.6177350893358</v>
       </c>
       <c r="E42" s="12" t="n">
         <f aca="false">E41-E20</f>
-        <v>22.5584906198161</v>
+        <v>22.6164554857076</v>
       </c>
       <c r="F42" s="12" t="n">
         <f aca="false">F41-F20</f>
-        <v>22.9576596665357</v>
+        <v>23.0156245324272</v>
       </c>
       <c r="G42" s="13" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="4" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B43" s="16" t="s">
         <v>69</v>
       </c>
       <c r="C43" s="22" t="n">
         <f aca="false">MAX(0,C16*cp*(C42-C40))</f>
-        <v>66.157941270466</v>
+        <v>66.9354433382906</v>
       </c>
       <c r="D43" s="22" t="n">
         <f aca="false">MAX(0,D16*cp*(D42-D40))</f>
-        <v>60.3653012637993</v>
+        <v>61.142803331624</v>
       </c>
       <c r="E43" s="22" t="n">
         <f aca="false">MAX(0,E16*cp*(E42-E40))</f>
-        <v>60.3481375137993</v>
+        <v>61.125639581624</v>
       </c>
       <c r="F43" s="22" t="n">
         <f aca="false">MAX(0,F16*cp*(F42-F40))</f>
-        <v>67.630491660466</v>
+        <v>68.4079937282906</v>
       </c>
       <c r="G43" s="13" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="4" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="B44" s="16" t="s">
         <v>69</v>
@@ -4937,12 +5001,12 @@
         <v>123.584619796667</v>
       </c>
       <c r="G44" s="13" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="23" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B45" s="16" t="s">
         <v>69</v>
@@ -4964,12 +5028,12 @@
         <v>140</v>
       </c>
       <c r="G45" s="13" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="3" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="B46" s="27"/>
       <c r="C46" s="27"/>
@@ -4980,7 +5044,7 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="4" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="B47" s="16" t="s">
         <v>69</v>
@@ -5005,7 +5069,7 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="4" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="B48" s="16" t="s">
         <v>69</v>
@@ -5030,7 +5094,7 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="4" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="B49" s="16" t="s">
         <v>69</v>
@@ -5052,12 +5116,12 @@
         <v>175</v>
       </c>
       <c r="G49" s="13" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="4" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="B50" s="16" t="s">
         <v>43</v>
@@ -5079,12 +5143,12 @@
         <v>2</v>
       </c>
       <c r="G50" s="13" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="4" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="B51" s="16" t="s">
         <v>69</v>
@@ -5109,7 +5173,7 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="4" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="B52" s="16" t="s">
         <v>69</v>
@@ -5134,7 +5198,7 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="3" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="B53" s="27"/>
       <c r="C53" s="27"/>
@@ -5145,7 +5209,7 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="4" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B54" s="16" t="s">
         <v>69</v>
@@ -5167,12 +5231,12 @@
         <v>200</v>
       </c>
       <c r="G54" s="13" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="4" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="B55" s="16" t="s">
         <v>11</v>
@@ -5194,12 +5258,12 @@
         <v>1.5</v>
       </c>
       <c r="G55" s="13" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="23" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="B56" s="16" t="s">
         <v>69</v>
@@ -5211,7 +5275,7 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="23" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="B57" s="16" t="s">
         <v>69</v>
@@ -5223,7 +5287,7 @@
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="23" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="B58" s="16" t="s">
         <v>69</v>
@@ -5259,36 +5323,36 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="B6" s="32" t="n">
         <v>40</v>
@@ -5297,12 +5361,12 @@
         <v>20</v>
       </c>
       <c r="D6" s="13" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="B7" s="32" t="n">
         <v>100</v>
@@ -5314,7 +5378,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="B8" s="32" t="n">
         <v>120</v>
@@ -5326,7 +5390,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="B9" s="32" t="n">
         <v>10</v>
@@ -5338,7 +5402,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="B10" s="32" t="n">
         <v>150</v>
@@ -5350,7 +5414,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="13" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="B11" s="32" t="n">
         <v>130</v>
@@ -5362,7 +5426,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="13" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="B12" s="32" t="n">
         <v>50</v>
@@ -5374,7 +5438,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="13" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="B13" s="32" t="n">
         <v>40</v>
@@ -5384,7 +5448,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="13" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="B14" s="32" t="n">
         <v>50</v>
@@ -5394,7 +5458,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="B15" s="34" t="n">
         <f aca="false">SUM(B6:B14)</f>
@@ -5410,12 +5474,12 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="3" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="B17" s="34" t="n">
         <f aca="false">0.6*v_ana^2</f>
@@ -5426,12 +5490,12 @@
         <v>19.97574</v>
       </c>
       <c r="D17" s="13" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="B18" s="34" t="n">
         <f aca="false">L_kr*R_ort</f>
@@ -5447,7 +5511,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="B19" s="34" t="n">
         <f aca="false">z_uf*B17</f>
@@ -5463,7 +5527,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="B20" s="34" t="n">
         <f aca="false">dp_mu+dp_br+dp_yd</f>
@@ -5479,7 +5543,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="B21" s="34" t="n">
         <f aca="false">SUM(B18:B20)</f>
@@ -5495,7 +5559,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="9" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="B22" s="35" t="n">
         <f aca="false">CEILING(B21,50)</f>
@@ -5511,7 +5575,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="23" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="B23" s="36" t="n">
         <f aca="false">B15+B22</f>
@@ -5522,17 +5586,17 @@
         <v>620</v>
       </c>
       <c r="D23" s="13" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="3" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="B25" s="34" t="n">
         <f aca="false">V_ks</f>
@@ -5543,36 +5607,36 @@
         <v>40000</v>
       </c>
       <c r="D25" s="13" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="B26" s="34" t="n">
         <f aca="false">n_fan</f>
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C26" s="34" t="n">
         <f aca="false">n_fan</f>
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D26" s="13" t="s">
-        <v>43</v>
+        <v>277</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="B27" s="34" t="n">
         <f aca="false">B25/B26</f>
-        <v>10000</v>
+        <v>40000</v>
       </c>
       <c r="C27" s="34" t="n">
         <f aca="false">C25/C26</f>
-        <v>10000</v>
+        <v>40000</v>
       </c>
       <c r="D27" s="13" t="s">
         <v>21</v>
@@ -5580,31 +5644,31 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="B28" s="28" t="n">
         <f aca="false">B25/3600*B23/eta_fan/1000</f>
-        <v>16.8458781362007</v>
+        <v>16.0683760683761</v>
       </c>
       <c r="C28" s="28" t="n">
         <f aca="false">C25/3600*C23/eta_fan/1000</f>
-        <v>11.1111111111111</v>
+        <v>10.5982905982906</v>
       </c>
       <c r="D28" s="13" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="B29" s="28" t="n">
         <f aca="false">B28/B26</f>
-        <v>4.21146953405018</v>
+        <v>16.0683760683761</v>
       </c>
       <c r="C29" s="28" t="n">
         <f aca="false">C28/C26</f>
-        <v>2.77777777777778</v>
+        <v>10.5982905982906</v>
       </c>
       <c r="D29" s="13" t="s">
         <v>69</v>
@@ -5612,55 +5676,55 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="9" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="B30" s="37" t="n">
-        <f aca="false">INDEX({1.1,1.5,2.2,3,4,5.5,7.5,11,15,18.5,22},MATCH(TRUE(),INDEX({1.1,1.5,2.2,3,4,5.5,7.5,11,15,18.5,22}&gt;=B29*k_motor,0),0))</f>
-        <v>5.5</v>
+        <f aca="false">INDEX({1.1,1.5,2.2,3,4,5.5,7.5,11,15,18.5,22,30,37,45},MATCH(TRUE(),INDEX({1.1,1.5,2.2,3,4,5.5,7.5,11,15,18.5,22,30,37,45}&gt;=B29*k_motor,0),0))</f>
+        <v>18.5</v>
       </c>
       <c r="C30" s="37" t="n">
-        <f aca="false">INDEX({1.1,1.5,2.2,3,4,5.5,7.5,11,15,18.5,22},MATCH(TRUE(),INDEX({1.1,1.5,2.2,3,4,5.5,7.5,11,15,18.5,22}&gt;=C29*k_motor,0),0))</f>
-        <v>4</v>
+        <f aca="false">INDEX({1.1,1.5,2.2,3,4,5.5,7.5,11,15,18.5,22,30,37,45},MATCH(TRUE(),INDEX({1.1,1.5,2.2,3,4,5.5,7.5,11,15,18.5,22,30,37,45}&gt;=C29*k_motor,0),0))</f>
+        <v>15</v>
       </c>
       <c r="D30" s="13" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="23" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="B31" s="38" t="n">
         <f aca="false">B26*B30</f>
-        <v>22</v>
+        <v>18.5</v>
       </c>
       <c r="C31" s="38" t="n">
         <f aca="false">C26*C30</f>
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D31" s="13" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="4" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="B32" s="34" t="n">
         <f aca="false">B28*1000/(B25/3600)</f>
-        <v>1516.12903225806</v>
+        <v>1446.15384615385</v>
       </c>
       <c r="C32" s="34" t="n">
         <f aca="false">C28*1000/(C25/3600)</f>
-        <v>1000</v>
+        <v>953.846153846154</v>
       </c>
       <c r="D32" s="13" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="4" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="B33" s="39" t="str">
         <f aca="false">IF(B32&lt;=500,"SFP1",IF(B32&lt;=750,"SFP2",IF(B32&lt;=1250,"SFP3",IF(B32&lt;=2000,"SFP4",IF(B32&lt;=3000,"SFP5","SFP6")))))</f>
@@ -5671,23 +5735,23 @@
         <v>SFP3</v>
       </c>
       <c r="D33" s="13" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="4" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="B34" s="28" t="n">
         <f aca="false">B28</f>
-        <v>16.8458781362007</v>
+        <v>16.0683760683761</v>
       </c>
       <c r="C34" s="28" t="n">
         <f aca="false">C28</f>
-        <v>11.1111111111111</v>
+        <v>10.5982905982906</v>
       </c>
       <c r="D34" s="13" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
     </row>
   </sheetData>
@@ -5718,44 +5782,44 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="H3" s="8" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="15" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="D4" s="19" t="n">
         <f aca="false">'KS HESABI'!C15</f>
@@ -5780,10 +5844,10 @@
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="15"/>
       <c r="B5" s="9" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="D5" s="19" t="n">
         <f aca="false">'KS HESABI'!C17</f>
@@ -5835,7 +5899,7 @@
       <c r="A7" s="15"/>
       <c r="B7" s="4"/>
       <c r="C7" s="4" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="D7" s="22" t="n">
         <f aca="false">'KS HESABI'!C37</f>
@@ -5854,14 +5918,14 @@
         <v>300</v>
       </c>
       <c r="H7" s="16" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="15"/>
       <c r="B8" s="4"/>
       <c r="C8" s="4" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="D8" s="22" t="n">
         <f aca="false">'KS HESABI'!C45</f>
@@ -5880,14 +5944,14 @@
         <v>140</v>
       </c>
       <c r="H8" s="16" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="15"/>
       <c r="B9" s="4"/>
       <c r="C9" s="4" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="D9" s="19" t="n">
         <f aca="false">'KS HESABI'!C36</f>
@@ -5906,38 +5970,40 @@
         <v>139.9624842906</v>
       </c>
       <c r="H9" s="16" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="15"/>
       <c r="B10" s="4"/>
       <c r="C10" s="4" t="s">
-        <v>301</v>
-      </c>
-      <c r="D10" s="19" t="str">
-        <f aca="false">n_fan&amp;" × "&amp;TEXT(qf_fan,"#.##0")&amp;" m³/h"</f>
-        <v>4 × 10000.000 m³/h</v>
-      </c>
-      <c r="E10" s="19" t="str">
-        <f aca="false">n_fan&amp;" × "&amp;TEXT(qf_fan,"#.##0")&amp;" m³/h"</f>
-        <v>4 × 10000.000 m³/h</v>
-      </c>
-      <c r="F10" s="19" t="str">
-        <f aca="false">n_fan&amp;" × "&amp;TEXT(qf_fan,"#.##0")&amp;" m³/h"</f>
-        <v>4 × 10000.000 m³/h</v>
-      </c>
-      <c r="G10" s="19" t="str">
-        <f aca="false">n_fan&amp;" × "&amp;TEXT(qf_fan,"#.##0")&amp;" m³/h"</f>
-        <v>4 × 10000.000 m³/h</v>
-      </c>
-      <c r="H10" s="16"/>
+        <v>303</v>
+      </c>
+      <c r="D10" s="19" t="n">
+        <f aca="false">qf_fan</f>
+        <v>40000</v>
+      </c>
+      <c r="E10" s="19" t="n">
+        <f aca="false">qf_fan</f>
+        <v>40000</v>
+      </c>
+      <c r="F10" s="19" t="n">
+        <f aca="false">qf_fan</f>
+        <v>40000</v>
+      </c>
+      <c r="G10" s="19" t="n">
+        <f aca="false">qf_fan</f>
+        <v>40000</v>
+      </c>
+      <c r="H10" s="16" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="15"/>
       <c r="B11" s="4"/>
       <c r="C11" s="4" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="D11" s="19" t="str">
         <f aca="false">TEXT(dp_uf,"0")&amp;" / "&amp;TEXT(esp_uf,"0")&amp;" Pa"</f>
@@ -5961,57 +6027,59 @@
       <c r="A12" s="15"/>
       <c r="B12" s="4"/>
       <c r="C12" s="4" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="D12" s="22" t="n">
         <f aca="false">Pm_uf</f>
-        <v>5.5</v>
+        <v>18.5</v>
       </c>
       <c r="E12" s="22" t="n">
         <f aca="false">Pm_uf</f>
-        <v>5.5</v>
+        <v>18.5</v>
       </c>
       <c r="F12" s="22" t="n">
         <f aca="false">Pm_uf</f>
-        <v>5.5</v>
+        <v>18.5</v>
       </c>
       <c r="G12" s="22" t="n">
         <f aca="false">Pm_uf</f>
-        <v>5.5</v>
+        <v>18.5</v>
       </c>
       <c r="H12" s="16" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="15"/>
       <c r="B13" s="4"/>
       <c r="C13" s="4" t="s">
-        <v>305</v>
-      </c>
-      <c r="D13" s="19" t="str">
-        <f aca="false">n_fan&amp;" × "&amp;TEXT(qf_fan,"#.##0")&amp;" m³/h"</f>
-        <v>4 × 10000.000 m³/h</v>
-      </c>
-      <c r="E13" s="19" t="str">
-        <f aca="false">n_fan&amp;" × "&amp;TEXT(qf_fan,"#.##0")&amp;" m³/h"</f>
-        <v>4 × 10000.000 m³/h</v>
-      </c>
-      <c r="F13" s="19" t="str">
-        <f aca="false">n_fan&amp;" × "&amp;TEXT(qf_fan,"#.##0")&amp;" m³/h"</f>
-        <v>4 × 10000.000 m³/h</v>
-      </c>
-      <c r="G13" s="19" t="str">
-        <f aca="false">n_fan&amp;" × "&amp;TEXT(qf_fan,"#.##0")&amp;" m³/h"</f>
-        <v>4 × 10000.000 m³/h</v>
-      </c>
-      <c r="H13" s="16"/>
+        <v>307</v>
+      </c>
+      <c r="D13" s="19" t="n">
+        <f aca="false">qf_fan</f>
+        <v>40000</v>
+      </c>
+      <c r="E13" s="19" t="n">
+        <f aca="false">qf_fan</f>
+        <v>40000</v>
+      </c>
+      <c r="F13" s="19" t="n">
+        <f aca="false">qf_fan</f>
+        <v>40000</v>
+      </c>
+      <c r="G13" s="19" t="n">
+        <f aca="false">qf_fan</f>
+        <v>40000</v>
+      </c>
+      <c r="H13" s="16" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="15"/>
       <c r="B14" s="4"/>
       <c r="C14" s="4" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="D14" s="19" t="str">
         <f aca="false">TEXT(dp_do,"0")&amp;" / "&amp;TEXT(esp_do,"0")&amp;" Pa"</f>
@@ -6035,49 +6103,49 @@
       <c r="A15" s="15"/>
       <c r="B15" s="4"/>
       <c r="C15" s="4" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="D15" s="22" t="n">
         <f aca="false">Pm_do</f>
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="E15" s="22" t="n">
         <f aca="false">Pm_do</f>
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="F15" s="22" t="n">
         <f aca="false">Pm_do</f>
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="G15" s="22" t="n">
         <f aca="false">Pm_do</f>
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="H15" s="16" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="15"/>
       <c r="B16" s="4"/>
       <c r="C16" s="4" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="D16" s="19" t="str">
         <f aca="false">TEXT(sfp_uf,"0")&amp;" / "&amp;TEXT(sfp_do,"0")&amp;" W/(m³/s)"</f>
-        <v>1516 / 1000 W/(m³/s)</v>
+        <v>1446 / 954 W/(m³/s)</v>
       </c>
       <c r="E16" s="19" t="str">
         <f aca="false">TEXT(sfp_uf,"0")&amp;" / "&amp;TEXT(sfp_do,"0")&amp;" W/(m³/s)"</f>
-        <v>1516 / 1000 W/(m³/s)</v>
+        <v>1446 / 954 W/(m³/s)</v>
       </c>
       <c r="F16" s="19" t="str">
         <f aca="false">TEXT(sfp_uf,"0")&amp;" / "&amp;TEXT(sfp_do,"0")&amp;" W/(m³/s)"</f>
-        <v>1516 / 1000 W/(m³/s)</v>
+        <v>1446 / 954 W/(m³/s)</v>
       </c>
       <c r="G16" s="19" t="str">
         <f aca="false">TEXT(sfp_uf,"0")&amp;" / "&amp;TEXT(sfp_do,"0")&amp;" W/(m³/s)"</f>
-        <v>1516 / 1000 W/(m³/s)</v>
+        <v>1446 / 954 W/(m³/s)</v>
       </c>
       <c r="H16" s="16"/>
     </row>
@@ -6085,19 +6153,19 @@
       <c r="A17" s="15"/>
       <c r="B17" s="4"/>
       <c r="C17" s="4" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="D17" s="19" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="E17" s="19" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="F17" s="19" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="G17" s="19" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="H17" s="16"/>
     </row>
@@ -6105,33 +6173,33 @@
       <c r="A18" s="15"/>
       <c r="B18" s="4"/>
       <c r="C18" s="4" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="D18" s="19" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="E18" s="19" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="F18" s="19" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="G18" s="19" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="H18" s="16" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="15" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="B19" s="9" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="D19" s="19" t="n">
         <f aca="false">'KS HESABI'!C50</f>
@@ -6157,7 +6225,7 @@
       <c r="A20" s="15"/>
       <c r="B20" s="4"/>
       <c r="C20" s="4" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="D20" s="22" t="n">
         <f aca="false">'KS HESABI'!C51</f>
@@ -6176,14 +6244,14 @@
         <v>150</v>
       </c>
       <c r="H20" s="16" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="15"/>
       <c r="B21" s="4"/>
       <c r="C21" s="4" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="D21" s="22" t="n">
         <f aca="false">'KS HESABI'!C52</f>
@@ -6202,34 +6270,34 @@
         <v>90</v>
       </c>
       <c r="H21" s="16" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="15"/>
       <c r="B22" s="4"/>
       <c r="C22" s="4" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="D22" s="19" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="E22" s="19" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="F22" s="19" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="G22" s="19" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="H22" s="16" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="2" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
     </row>
   </sheetData>
@@ -6264,44 +6332,44 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="14" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="E4" s="14" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="F4" s="14" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="G4" s="14" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="H4" s="14" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="I4" s="14" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="J4" s="14" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6309,16 +6377,21 @@
         <v>1</v>
       </c>
       <c r="B5" s="41" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C5" s="23" t="s">
-        <v>333</v>
-      </c>
-      <c r="D5" s="36"/>
-      <c r="E5" s="38"/>
+        <v>335</v>
+      </c>
+      <c r="D5" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" s="42" t="n">
+        <f aca="false">SUM(F6:F9)</f>
+        <v>33.666</v>
+      </c>
       <c r="F5" s="38" t="n">
-        <f aca="false">SUM(F6:F9)</f>
-        <v>38.34</v>
+        <f aca="false">D5*E5</f>
+        <v>33.666</v>
       </c>
       <c r="G5" s="36" t="n">
         <f aca="false">U_v</f>
@@ -6328,9 +6401,9 @@
         <f aca="false">cos_ks</f>
         <v>0.95</v>
       </c>
-      <c r="I5" s="42" t="n">
+      <c r="I5" s="43" t="n">
         <f aca="false">F5*1000/(SQRT(3)*G5*H5)</f>
-        <v>58.2516034756059</v>
+        <v>51.1501951645735</v>
       </c>
       <c r="J5" s="36" t="n">
         <f aca="false">INDEX({6,10,16,20,25,32,40,50,63,80,100,125,160,200,250},MATCH(TRUE(),INDEX({6,10,16,20,25,32,40,50,63,80,100,125,160,200,250}&gt;=I5*k_sig,0),0))</f>
@@ -6339,23 +6412,25 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="16" t="s">
-        <v>334</v>
-      </c>
-      <c r="B6" s="16"/>
+        <v>336</v>
+      </c>
+      <c r="B6" s="16" t="s">
+        <v>337</v>
+      </c>
       <c r="C6" s="4" t="s">
-        <v>335</v>
+        <v>338</v>
       </c>
       <c r="D6" s="34" t="n">
         <f aca="false">n_fan</f>
-        <v>4</v>
-      </c>
-      <c r="E6" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" s="44" t="n">
         <f aca="false">Pm_uf</f>
-        <v>5.5</v>
+        <v>18.5</v>
       </c>
       <c r="F6" s="28" t="n">
         <f aca="false">D6*E6</f>
-        <v>22</v>
+        <v>18.5</v>
       </c>
       <c r="G6" s="34" t="n">
         <f aca="false">U_v</f>
@@ -6367,32 +6442,34 @@
       </c>
       <c r="I6" s="12" t="n">
         <f aca="false">E6*1000/(SQRT(3)*G6*H6)</f>
-        <v>8.356385475113</v>
+        <v>28.1078420526528</v>
       </c>
       <c r="J6" s="34" t="n">
         <f aca="false">INDEX({6,10,16,20,25,32,40,50,63,80,100,125,160,200,250},MATCH(TRUE(),INDEX({6,10,16,20,25,32,40,50,63,80,100,125,160,200,250}&gt;=I6*k_sig,0),0))</f>
-        <v>16</v>
+        <v>40</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="16" t="s">
-        <v>336</v>
-      </c>
-      <c r="B7" s="16"/>
+        <v>339</v>
+      </c>
+      <c r="B7" s="16" t="s">
+        <v>340</v>
+      </c>
       <c r="C7" s="4" t="s">
-        <v>337</v>
+        <v>341</v>
       </c>
       <c r="D7" s="34" t="n">
         <f aca="false">n_fan</f>
-        <v>4</v>
-      </c>
-      <c r="E7" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" s="44" t="n">
         <f aca="false">Pm_do</f>
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="F7" s="28" t="n">
         <f aca="false">D7*E7</f>
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G7" s="34" t="n">
         <f aca="false">U_v</f>
@@ -6404,31 +6481,33 @@
       </c>
       <c r="I7" s="12" t="n">
         <f aca="false">E7*1000/(SQRT(3)*G7*H7)</f>
-        <v>6.07737125462764</v>
+        <v>22.7901422048537</v>
       </c>
       <c r="J7" s="34" t="n">
         <f aca="false">INDEX({6,10,16,20,25,32,40,50,63,80,100,125,160,200,250},MATCH(TRUE(),INDEX({6,10,16,20,25,32,40,50,63,80,100,125,160,200,250}&gt;=I7*k_sig,0),0))</f>
-        <v>10</v>
+        <v>32</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="16" t="s">
-        <v>338</v>
-      </c>
-      <c r="B8" s="16"/>
+        <v>342</v>
+      </c>
+      <c r="B8" s="16" t="s">
+        <v>343</v>
+      </c>
       <c r="C8" s="4" t="s">
-        <v>339</v>
+        <v>344</v>
       </c>
       <c r="D8" s="34" t="n">
         <v>4</v>
       </c>
-      <c r="E8" s="28" t="n">
+      <c r="E8" s="44" t="n">
         <f aca="false">P_dmp</f>
-        <v>0.01</v>
+        <v>0.004</v>
       </c>
       <c r="F8" s="28" t="n">
         <f aca="false">D8*E8</f>
-        <v>0.04</v>
+        <v>0.016</v>
       </c>
       <c r="G8" s="34" t="n">
         <v>230</v>
@@ -6439,7 +6518,7 @@
       </c>
       <c r="I8" s="12" t="n">
         <f aca="false">F8*1000/(G8*H8)</f>
-        <v>0.183066361556064</v>
+        <v>0.0732265446224256</v>
       </c>
       <c r="J8" s="34" t="n">
         <f aca="false">INDEX({6,10,16,20,25,32,40,50,63,80,100,125,160,200,250},MATCH(TRUE(),INDEX({6,10,16,20,25,32,40,50,63,80,100,125,160,200,250}&gt;=I8*k_sig,0),0))</f>
@@ -6448,22 +6527,24 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="16" t="s">
-        <v>340</v>
-      </c>
-      <c r="B9" s="16"/>
+        <v>345</v>
+      </c>
+      <c r="B9" s="16" t="s">
+        <v>346</v>
+      </c>
       <c r="C9" s="4" t="s">
-        <v>341</v>
+        <v>347</v>
       </c>
       <c r="D9" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="E9" s="28" t="n">
+      <c r="E9" s="44" t="n">
         <f aca="false">P_ddc</f>
-        <v>0.3</v>
+        <v>0.15</v>
       </c>
       <c r="F9" s="28" t="n">
         <f aca="false">D9*E9</f>
-        <v>0.3</v>
+        <v>0.15</v>
       </c>
       <c r="G9" s="34" t="n">
         <v>230</v>
@@ -6474,7 +6555,7 @@
       </c>
       <c r="I9" s="12" t="n">
         <f aca="false">F9*1000/(G9*H9)</f>
-        <v>1.37299771167048</v>
+        <v>0.68649885583524</v>
       </c>
       <c r="J9" s="34" t="n">
         <f aca="false">INDEX({6,10,16,20,25,32,40,50,63,80,100,125,160,200,250},MATCH(TRUE(),INDEX({6,10,16,20,25,32,40,50,63,80,100,125,160,200,250}&gt;=I9*k_sig,0),0))</f>
@@ -6486,21 +6567,21 @@
         <v>2</v>
       </c>
       <c r="B10" s="41" t="s">
-        <v>342</v>
+        <v>348</v>
       </c>
       <c r="C10" s="23" t="s">
-        <v>343</v>
+        <v>349</v>
       </c>
       <c r="D10" s="36" t="n">
         <v>1</v>
       </c>
-      <c r="E10" s="38" t="n">
+      <c r="E10" s="42" t="n">
         <f aca="false">ROUND(MAX('KS HESABI'!C51/EER,'KS HESABI'!C52*dus/COP),1)</f>
-        <v>50</v>
+        <v>53.6</v>
       </c>
       <c r="F10" s="38" t="n">
         <f aca="false">D10*E10</f>
-        <v>50</v>
+        <v>53.6</v>
       </c>
       <c r="G10" s="36" t="n">
         <f aca="false">U_v</f>
@@ -6510,13 +6591,13 @@
         <f aca="false">cos_du</f>
         <v>0.92</v>
       </c>
-      <c r="I10" s="42" t="n">
+      <c r="I10" s="43" t="n">
         <f aca="false">F10*1000/(SQRT(3)*G10*H10)</f>
-        <v>78.4443300529383</v>
+        <v>84.0923218167498</v>
       </c>
       <c r="J10" s="36" t="n">
         <f aca="false">INDEX({6,10,16,20,25,32,40,50,63,80,100,125,160,200,250},MATCH(TRUE(),INDEX({6,10,16,20,25,32,40,50,63,80,100,125,160,200,250}&gt;=I10*k_sig,0),0))</f>
-        <v>100</v>
+        <v>125</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6524,21 +6605,21 @@
         <v>3</v>
       </c>
       <c r="B11" s="41" t="s">
-        <v>344</v>
+        <v>350</v>
       </c>
       <c r="C11" s="23" t="s">
-        <v>343</v>
+        <v>349</v>
       </c>
       <c r="D11" s="36" t="n">
         <v>1</v>
       </c>
-      <c r="E11" s="38" t="n">
+      <c r="E11" s="42" t="n">
         <f aca="false">ROUND(MAX('KS HESABI'!C51/EER,'KS HESABI'!C52*dus/COP),1)</f>
-        <v>50</v>
+        <v>53.6</v>
       </c>
       <c r="F11" s="38" t="n">
         <f aca="false">D11*E11</f>
-        <v>50</v>
+        <v>53.6</v>
       </c>
       <c r="G11" s="36" t="n">
         <f aca="false">U_v</f>
@@ -6548,13 +6629,13 @@
         <f aca="false">cos_du</f>
         <v>0.92</v>
       </c>
-      <c r="I11" s="42" t="n">
+      <c r="I11" s="43" t="n">
         <f aca="false">F11*1000/(SQRT(3)*G11*H11)</f>
-        <v>78.4443300529383</v>
+        <v>84.0923218167498</v>
       </c>
       <c r="J11" s="36" t="n">
         <f aca="false">INDEX({6,10,16,20,25,32,40,50,63,80,100,125,160,200,250},MATCH(TRUE(),INDEX({6,10,16,20,25,32,40,50,63,80,100,125,160,200,250}&gt;=I11*k_sig,0),0))</f>
-        <v>100</v>
+        <v>125</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6562,16 +6643,21 @@
         <v>4</v>
       </c>
       <c r="B12" s="41" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C12" s="23" t="s">
-        <v>333</v>
-      </c>
-      <c r="D12" s="36"/>
-      <c r="E12" s="38"/>
+        <v>335</v>
+      </c>
+      <c r="D12" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" s="42" t="n">
+        <f aca="false">SUM(F13:F16)</f>
+        <v>33.666</v>
+      </c>
       <c r="F12" s="38" t="n">
-        <f aca="false">SUM(F13:F16)</f>
-        <v>38.34</v>
+        <f aca="false">D12*E12</f>
+        <v>33.666</v>
       </c>
       <c r="G12" s="36" t="n">
         <f aca="false">U_v</f>
@@ -6581,9 +6667,9 @@
         <f aca="false">cos_ks</f>
         <v>0.95</v>
       </c>
-      <c r="I12" s="42" t="n">
+      <c r="I12" s="43" t="n">
         <f aca="false">F12*1000/(SQRT(3)*G12*H12)</f>
-        <v>58.2516034756059</v>
+        <v>51.1501951645735</v>
       </c>
       <c r="J12" s="36" t="n">
         <f aca="false">INDEX({6,10,16,20,25,32,40,50,63,80,100,125,160,200,250},MATCH(TRUE(),INDEX({6,10,16,20,25,32,40,50,63,80,100,125,160,200,250}&gt;=I12*k_sig,0),0))</f>
@@ -6592,23 +6678,25 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="16" t="s">
-        <v>345</v>
-      </c>
-      <c r="B13" s="16"/>
+        <v>351</v>
+      </c>
+      <c r="B13" s="16" t="s">
+        <v>352</v>
+      </c>
       <c r="C13" s="4" t="s">
-        <v>335</v>
+        <v>338</v>
       </c>
       <c r="D13" s="34" t="n">
         <f aca="false">n_fan</f>
-        <v>4</v>
-      </c>
-      <c r="E13" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" s="44" t="n">
         <f aca="false">Pm_uf</f>
-        <v>5.5</v>
+        <v>18.5</v>
       </c>
       <c r="F13" s="28" t="n">
         <f aca="false">D13*E13</f>
-        <v>22</v>
+        <v>18.5</v>
       </c>
       <c r="G13" s="34" t="n">
         <f aca="false">U_v</f>
@@ -6620,32 +6708,34 @@
       </c>
       <c r="I13" s="12" t="n">
         <f aca="false">E13*1000/(SQRT(3)*G13*H13)</f>
-        <v>8.356385475113</v>
+        <v>28.1078420526528</v>
       </c>
       <c r="J13" s="34" t="n">
         <f aca="false">INDEX({6,10,16,20,25,32,40,50,63,80,100,125,160,200,250},MATCH(TRUE(),INDEX({6,10,16,20,25,32,40,50,63,80,100,125,160,200,250}&gt;=I13*k_sig,0),0))</f>
-        <v>16</v>
+        <v>40</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="16" t="s">
-        <v>346</v>
-      </c>
-      <c r="B14" s="16"/>
+        <v>353</v>
+      </c>
+      <c r="B14" s="16" t="s">
+        <v>354</v>
+      </c>
       <c r="C14" s="4" t="s">
-        <v>337</v>
+        <v>341</v>
       </c>
       <c r="D14" s="34" t="n">
         <f aca="false">n_fan</f>
-        <v>4</v>
-      </c>
-      <c r="E14" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" s="44" t="n">
         <f aca="false">Pm_do</f>
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="F14" s="28" t="n">
         <f aca="false">D14*E14</f>
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G14" s="34" t="n">
         <f aca="false">U_v</f>
@@ -6657,31 +6747,33 @@
       </c>
       <c r="I14" s="12" t="n">
         <f aca="false">E14*1000/(SQRT(3)*G14*H14)</f>
-        <v>6.07737125462764</v>
+        <v>22.7901422048537</v>
       </c>
       <c r="J14" s="34" t="n">
         <f aca="false">INDEX({6,10,16,20,25,32,40,50,63,80,100,125,160,200,250},MATCH(TRUE(),INDEX({6,10,16,20,25,32,40,50,63,80,100,125,160,200,250}&gt;=I14*k_sig,0),0))</f>
-        <v>10</v>
+        <v>32</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="16" t="s">
-        <v>347</v>
-      </c>
-      <c r="B15" s="16"/>
+        <v>355</v>
+      </c>
+      <c r="B15" s="16" t="s">
+        <v>356</v>
+      </c>
       <c r="C15" s="4" t="s">
-        <v>339</v>
+        <v>344</v>
       </c>
       <c r="D15" s="34" t="n">
         <v>4</v>
       </c>
-      <c r="E15" s="28" t="n">
+      <c r="E15" s="44" t="n">
         <f aca="false">P_dmp</f>
-        <v>0.01</v>
+        <v>0.004</v>
       </c>
       <c r="F15" s="28" t="n">
         <f aca="false">D15*E15</f>
-        <v>0.04</v>
+        <v>0.016</v>
       </c>
       <c r="G15" s="34" t="n">
         <v>230</v>
@@ -6692,7 +6784,7 @@
       </c>
       <c r="I15" s="12" t="n">
         <f aca="false">F15*1000/(G15*H15)</f>
-        <v>0.183066361556064</v>
+        <v>0.0732265446224256</v>
       </c>
       <c r="J15" s="34" t="n">
         <f aca="false">INDEX({6,10,16,20,25,32,40,50,63,80,100,125,160,200,250},MATCH(TRUE(),INDEX({6,10,16,20,25,32,40,50,63,80,100,125,160,200,250}&gt;=I15*k_sig,0),0))</f>
@@ -6701,22 +6793,24 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="16" t="s">
-        <v>348</v>
-      </c>
-      <c r="B16" s="16"/>
+        <v>357</v>
+      </c>
+      <c r="B16" s="16" t="s">
+        <v>358</v>
+      </c>
       <c r="C16" s="4" t="s">
-        <v>341</v>
+        <v>347</v>
       </c>
       <c r="D16" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="E16" s="28" t="n">
+      <c r="E16" s="44" t="n">
         <f aca="false">P_ddc</f>
-        <v>0.3</v>
+        <v>0.15</v>
       </c>
       <c r="F16" s="28" t="n">
         <f aca="false">D16*E16</f>
-        <v>0.3</v>
+        <v>0.15</v>
       </c>
       <c r="G16" s="34" t="n">
         <v>230</v>
@@ -6727,7 +6821,7 @@
       </c>
       <c r="I16" s="12" t="n">
         <f aca="false">F16*1000/(G16*H16)</f>
-        <v>1.37299771167048</v>
+        <v>0.68649885583524</v>
       </c>
       <c r="J16" s="34" t="n">
         <f aca="false">INDEX({6,10,16,20,25,32,40,50,63,80,100,125,160,200,250},MATCH(TRUE(),INDEX({6,10,16,20,25,32,40,50,63,80,100,125,160,200,250}&gt;=I16*k_sig,0),0))</f>
@@ -6739,21 +6833,21 @@
         <v>5</v>
       </c>
       <c r="B17" s="41" t="s">
+        <v>359</v>
+      </c>
+      <c r="C17" s="23" t="s">
         <v>349</v>
-      </c>
-      <c r="C17" s="23" t="s">
-        <v>343</v>
       </c>
       <c r="D17" s="36" t="n">
         <v>1</v>
       </c>
-      <c r="E17" s="38" t="n">
+      <c r="E17" s="42" t="n">
         <f aca="false">ROUND(MAX('KS HESABI'!D51/EER,'KS HESABI'!D52*dus/COP),1)</f>
-        <v>46.7</v>
+        <v>50</v>
       </c>
       <c r="F17" s="38" t="n">
         <f aca="false">D17*E17</f>
-        <v>46.7</v>
+        <v>50</v>
       </c>
       <c r="G17" s="36" t="n">
         <f aca="false">U_v</f>
@@ -6763,9 +6857,9 @@
         <f aca="false">cos_du</f>
         <v>0.92</v>
       </c>
-      <c r="I17" s="42" t="n">
+      <c r="I17" s="43" t="n">
         <f aca="false">F17*1000/(SQRT(3)*G17*H17)</f>
-        <v>73.2670042694444</v>
+        <v>78.4443300529383</v>
       </c>
       <c r="J17" s="36" t="n">
         <f aca="false">INDEX({6,10,16,20,25,32,40,50,63,80,100,125,160,200,250},MATCH(TRUE(),INDEX({6,10,16,20,25,32,40,50,63,80,100,125,160,200,250}&gt;=I17*k_sig,0),0))</f>
@@ -6777,21 +6871,21 @@
         <v>6</v>
       </c>
       <c r="B18" s="41" t="s">
-        <v>350</v>
+        <v>360</v>
       </c>
       <c r="C18" s="23" t="s">
-        <v>343</v>
+        <v>349</v>
       </c>
       <c r="D18" s="36" t="n">
         <v>1</v>
       </c>
-      <c r="E18" s="38" t="n">
+      <c r="E18" s="42" t="n">
         <f aca="false">ROUND(MAX('KS HESABI'!D51/EER,'KS HESABI'!D52*dus/COP),1)</f>
-        <v>46.7</v>
+        <v>50</v>
       </c>
       <c r="F18" s="38" t="n">
         <f aca="false">D18*E18</f>
-        <v>46.7</v>
+        <v>50</v>
       </c>
       <c r="G18" s="36" t="n">
         <f aca="false">U_v</f>
@@ -6801,9 +6895,9 @@
         <f aca="false">cos_du</f>
         <v>0.92</v>
       </c>
-      <c r="I18" s="42" t="n">
+      <c r="I18" s="43" t="n">
         <f aca="false">F18*1000/(SQRT(3)*G18*H18)</f>
-        <v>73.2670042694444</v>
+        <v>78.4443300529383</v>
       </c>
       <c r="J18" s="36" t="n">
         <f aca="false">INDEX({6,10,16,20,25,32,40,50,63,80,100,125,160,200,250},MATCH(TRUE(),INDEX({6,10,16,20,25,32,40,50,63,80,100,125,160,200,250}&gt;=I18*k_sig,0),0))</f>
@@ -6815,16 +6909,21 @@
         <v>7</v>
       </c>
       <c r="B19" s="41" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C19" s="23" t="s">
-        <v>333</v>
-      </c>
-      <c r="D19" s="36"/>
-      <c r="E19" s="38"/>
+        <v>335</v>
+      </c>
+      <c r="D19" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="E19" s="42" t="n">
+        <f aca="false">SUM(F20:F23)</f>
+        <v>33.666</v>
+      </c>
       <c r="F19" s="38" t="n">
-        <f aca="false">SUM(F20:F23)</f>
-        <v>38.34</v>
+        <f aca="false">D19*E19</f>
+        <v>33.666</v>
       </c>
       <c r="G19" s="36" t="n">
         <f aca="false">U_v</f>
@@ -6834,9 +6933,9 @@
         <f aca="false">cos_ks</f>
         <v>0.95</v>
       </c>
-      <c r="I19" s="42" t="n">
+      <c r="I19" s="43" t="n">
         <f aca="false">F19*1000/(SQRT(3)*G19*H19)</f>
-        <v>58.2516034756059</v>
+        <v>51.1501951645735</v>
       </c>
       <c r="J19" s="36" t="n">
         <f aca="false">INDEX({6,10,16,20,25,32,40,50,63,80,100,125,160,200,250},MATCH(TRUE(),INDEX({6,10,16,20,25,32,40,50,63,80,100,125,160,200,250}&gt;=I19*k_sig,0),0))</f>
@@ -6845,23 +6944,25 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="16" t="s">
-        <v>351</v>
-      </c>
-      <c r="B20" s="16"/>
+        <v>361</v>
+      </c>
+      <c r="B20" s="16" t="s">
+        <v>362</v>
+      </c>
       <c r="C20" s="4" t="s">
-        <v>335</v>
+        <v>338</v>
       </c>
       <c r="D20" s="34" t="n">
         <f aca="false">n_fan</f>
-        <v>4</v>
-      </c>
-      <c r="E20" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="E20" s="44" t="n">
         <f aca="false">Pm_uf</f>
-        <v>5.5</v>
+        <v>18.5</v>
       </c>
       <c r="F20" s="28" t="n">
         <f aca="false">D20*E20</f>
-        <v>22</v>
+        <v>18.5</v>
       </c>
       <c r="G20" s="34" t="n">
         <f aca="false">U_v</f>
@@ -6873,32 +6974,34 @@
       </c>
       <c r="I20" s="12" t="n">
         <f aca="false">E20*1000/(SQRT(3)*G20*H20)</f>
-        <v>8.356385475113</v>
+        <v>28.1078420526528</v>
       </c>
       <c r="J20" s="34" t="n">
         <f aca="false">INDEX({6,10,16,20,25,32,40,50,63,80,100,125,160,200,250},MATCH(TRUE(),INDEX({6,10,16,20,25,32,40,50,63,80,100,125,160,200,250}&gt;=I20*k_sig,0),0))</f>
-        <v>16</v>
+        <v>40</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="16" t="s">
-        <v>352</v>
-      </c>
-      <c r="B21" s="16"/>
+        <v>363</v>
+      </c>
+      <c r="B21" s="16" t="s">
+        <v>364</v>
+      </c>
       <c r="C21" s="4" t="s">
-        <v>337</v>
+        <v>341</v>
       </c>
       <c r="D21" s="34" t="n">
         <f aca="false">n_fan</f>
-        <v>4</v>
-      </c>
-      <c r="E21" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="E21" s="44" t="n">
         <f aca="false">Pm_do</f>
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="F21" s="28" t="n">
         <f aca="false">D21*E21</f>
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G21" s="34" t="n">
         <f aca="false">U_v</f>
@@ -6910,31 +7013,33 @@
       </c>
       <c r="I21" s="12" t="n">
         <f aca="false">E21*1000/(SQRT(3)*G21*H21)</f>
-        <v>6.07737125462764</v>
+        <v>22.7901422048537</v>
       </c>
       <c r="J21" s="34" t="n">
         <f aca="false">INDEX({6,10,16,20,25,32,40,50,63,80,100,125,160,200,250},MATCH(TRUE(),INDEX({6,10,16,20,25,32,40,50,63,80,100,125,160,200,250}&gt;=I21*k_sig,0),0))</f>
-        <v>10</v>
+        <v>32</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="16" t="s">
-        <v>353</v>
-      </c>
-      <c r="B22" s="16"/>
+        <v>365</v>
+      </c>
+      <c r="B22" s="16" t="s">
+        <v>366</v>
+      </c>
       <c r="C22" s="4" t="s">
-        <v>339</v>
+        <v>344</v>
       </c>
       <c r="D22" s="34" t="n">
         <v>4</v>
       </c>
-      <c r="E22" s="28" t="n">
+      <c r="E22" s="44" t="n">
         <f aca="false">P_dmp</f>
-        <v>0.01</v>
+        <v>0.004</v>
       </c>
       <c r="F22" s="28" t="n">
         <f aca="false">D22*E22</f>
-        <v>0.04</v>
+        <v>0.016</v>
       </c>
       <c r="G22" s="34" t="n">
         <v>230</v>
@@ -6945,7 +7050,7 @@
       </c>
       <c r="I22" s="12" t="n">
         <f aca="false">F22*1000/(G22*H22)</f>
-        <v>0.183066361556064</v>
+        <v>0.0732265446224256</v>
       </c>
       <c r="J22" s="34" t="n">
         <f aca="false">INDEX({6,10,16,20,25,32,40,50,63,80,100,125,160,200,250},MATCH(TRUE(),INDEX({6,10,16,20,25,32,40,50,63,80,100,125,160,200,250}&gt;=I22*k_sig,0),0))</f>
@@ -6954,22 +7059,24 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="16" t="s">
-        <v>354</v>
-      </c>
-      <c r="B23" s="16"/>
+        <v>367</v>
+      </c>
+      <c r="B23" s="16" t="s">
+        <v>368</v>
+      </c>
       <c r="C23" s="4" t="s">
-        <v>341</v>
+        <v>347</v>
       </c>
       <c r="D23" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="E23" s="28" t="n">
+      <c r="E23" s="44" t="n">
         <f aca="false">P_ddc</f>
-        <v>0.3</v>
+        <v>0.15</v>
       </c>
       <c r="F23" s="28" t="n">
         <f aca="false">D23*E23</f>
-        <v>0.3</v>
+        <v>0.15</v>
       </c>
       <c r="G23" s="34" t="n">
         <v>230</v>
@@ -6980,7 +7087,7 @@
       </c>
       <c r="I23" s="12" t="n">
         <f aca="false">F23*1000/(G23*H23)</f>
-        <v>1.37299771167048</v>
+        <v>0.68649885583524</v>
       </c>
       <c r="J23" s="34" t="n">
         <f aca="false">INDEX({6,10,16,20,25,32,40,50,63,80,100,125,160,200,250},MATCH(TRUE(),INDEX({6,10,16,20,25,32,40,50,63,80,100,125,160,200,250}&gt;=I23*k_sig,0),0))</f>
@@ -6992,21 +7099,21 @@
         <v>8</v>
       </c>
       <c r="B24" s="41" t="s">
-        <v>355</v>
+        <v>369</v>
       </c>
       <c r="C24" s="23" t="s">
-        <v>343</v>
+        <v>349</v>
       </c>
       <c r="D24" s="36" t="n">
         <v>1</v>
       </c>
-      <c r="E24" s="38" t="n">
+      <c r="E24" s="42" t="n">
         <f aca="false">ROUND(MAX('KS HESABI'!E51/EER,'KS HESABI'!E52*dus/COP),1)</f>
-        <v>46.7</v>
+        <v>50</v>
       </c>
       <c r="F24" s="38" t="n">
         <f aca="false">D24*E24</f>
-        <v>46.7</v>
+        <v>50</v>
       </c>
       <c r="G24" s="36" t="n">
         <f aca="false">U_v</f>
@@ -7016,9 +7123,9 @@
         <f aca="false">cos_du</f>
         <v>0.92</v>
       </c>
-      <c r="I24" s="42" t="n">
+      <c r="I24" s="43" t="n">
         <f aca="false">F24*1000/(SQRT(3)*G24*H24)</f>
-        <v>73.2670042694444</v>
+        <v>78.4443300529383</v>
       </c>
       <c r="J24" s="36" t="n">
         <f aca="false">INDEX({6,10,16,20,25,32,40,50,63,80,100,125,160,200,250},MATCH(TRUE(),INDEX({6,10,16,20,25,32,40,50,63,80,100,125,160,200,250}&gt;=I24*k_sig,0),0))</f>
@@ -7030,21 +7137,21 @@
         <v>9</v>
       </c>
       <c r="B25" s="41" t="s">
-        <v>356</v>
+        <v>370</v>
       </c>
       <c r="C25" s="23" t="s">
-        <v>343</v>
+        <v>349</v>
       </c>
       <c r="D25" s="36" t="n">
         <v>1</v>
       </c>
-      <c r="E25" s="38" t="n">
+      <c r="E25" s="42" t="n">
         <f aca="false">ROUND(MAX('KS HESABI'!E51/EER,'KS HESABI'!E52*dus/COP),1)</f>
-        <v>46.7</v>
+        <v>50</v>
       </c>
       <c r="F25" s="38" t="n">
         <f aca="false">D25*E25</f>
-        <v>46.7</v>
+        <v>50</v>
       </c>
       <c r="G25" s="36" t="n">
         <f aca="false">U_v</f>
@@ -7054,9 +7161,9 @@
         <f aca="false">cos_du</f>
         <v>0.92</v>
       </c>
-      <c r="I25" s="42" t="n">
+      <c r="I25" s="43" t="n">
         <f aca="false">F25*1000/(SQRT(3)*G25*H25)</f>
-        <v>73.2670042694444</v>
+        <v>78.4443300529383</v>
       </c>
       <c r="J25" s="36" t="n">
         <f aca="false">INDEX({6,10,16,20,25,32,40,50,63,80,100,125,160,200,250},MATCH(TRUE(),INDEX({6,10,16,20,25,32,40,50,63,80,100,125,160,200,250}&gt;=I25*k_sig,0),0))</f>
@@ -7068,16 +7175,21 @@
         <v>10</v>
       </c>
       <c r="B26" s="41" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C26" s="23" t="s">
-        <v>333</v>
-      </c>
-      <c r="D26" s="36"/>
-      <c r="E26" s="38"/>
+        <v>335</v>
+      </c>
+      <c r="D26" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="E26" s="42" t="n">
+        <f aca="false">SUM(F27:F30)</f>
+        <v>33.666</v>
+      </c>
       <c r="F26" s="38" t="n">
-        <f aca="false">SUM(F27:F30)</f>
-        <v>38.34</v>
+        <f aca="false">D26*E26</f>
+        <v>33.666</v>
       </c>
       <c r="G26" s="36" t="n">
         <f aca="false">U_v</f>
@@ -7087,9 +7199,9 @@
         <f aca="false">cos_ks</f>
         <v>0.95</v>
       </c>
-      <c r="I26" s="42" t="n">
+      <c r="I26" s="43" t="n">
         <f aca="false">F26*1000/(SQRT(3)*G26*H26)</f>
-        <v>58.2516034756059</v>
+        <v>51.1501951645735</v>
       </c>
       <c r="J26" s="36" t="n">
         <f aca="false">INDEX({6,10,16,20,25,32,40,50,63,80,100,125,160,200,250},MATCH(TRUE(),INDEX({6,10,16,20,25,32,40,50,63,80,100,125,160,200,250}&gt;=I26*k_sig,0),0))</f>
@@ -7098,23 +7210,25 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="16" t="s">
-        <v>357</v>
-      </c>
-      <c r="B27" s="16"/>
+        <v>371</v>
+      </c>
+      <c r="B27" s="16" t="s">
+        <v>372</v>
+      </c>
       <c r="C27" s="4" t="s">
-        <v>335</v>
+        <v>338</v>
       </c>
       <c r="D27" s="34" t="n">
         <f aca="false">n_fan</f>
-        <v>4</v>
-      </c>
-      <c r="E27" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="E27" s="44" t="n">
         <f aca="false">Pm_uf</f>
-        <v>5.5</v>
+        <v>18.5</v>
       </c>
       <c r="F27" s="28" t="n">
         <f aca="false">D27*E27</f>
-        <v>22</v>
+        <v>18.5</v>
       </c>
       <c r="G27" s="34" t="n">
         <f aca="false">U_v</f>
@@ -7126,32 +7240,34 @@
       </c>
       <c r="I27" s="12" t="n">
         <f aca="false">E27*1000/(SQRT(3)*G27*H27)</f>
-        <v>8.356385475113</v>
+        <v>28.1078420526528</v>
       </c>
       <c r="J27" s="34" t="n">
         <f aca="false">INDEX({6,10,16,20,25,32,40,50,63,80,100,125,160,200,250},MATCH(TRUE(),INDEX({6,10,16,20,25,32,40,50,63,80,100,125,160,200,250}&gt;=I27*k_sig,0),0))</f>
-        <v>16</v>
+        <v>40</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="16" t="s">
-        <v>358</v>
-      </c>
-      <c r="B28" s="16"/>
+        <v>373</v>
+      </c>
+      <c r="B28" s="16" t="s">
+        <v>374</v>
+      </c>
       <c r="C28" s="4" t="s">
-        <v>337</v>
+        <v>341</v>
       </c>
       <c r="D28" s="34" t="n">
         <f aca="false">n_fan</f>
-        <v>4</v>
-      </c>
-      <c r="E28" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="E28" s="44" t="n">
         <f aca="false">Pm_do</f>
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="F28" s="28" t="n">
         <f aca="false">D28*E28</f>
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G28" s="34" t="n">
         <f aca="false">U_v</f>
@@ -7163,31 +7279,33 @@
       </c>
       <c r="I28" s="12" t="n">
         <f aca="false">E28*1000/(SQRT(3)*G28*H28)</f>
-        <v>6.07737125462764</v>
+        <v>22.7901422048537</v>
       </c>
       <c r="J28" s="34" t="n">
         <f aca="false">INDEX({6,10,16,20,25,32,40,50,63,80,100,125,160,200,250},MATCH(TRUE(),INDEX({6,10,16,20,25,32,40,50,63,80,100,125,160,200,250}&gt;=I28*k_sig,0),0))</f>
-        <v>10</v>
+        <v>32</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="16" t="s">
-        <v>359</v>
-      </c>
-      <c r="B29" s="16"/>
+        <v>375</v>
+      </c>
+      <c r="B29" s="16" t="s">
+        <v>376</v>
+      </c>
       <c r="C29" s="4" t="s">
-        <v>339</v>
+        <v>344</v>
       </c>
       <c r="D29" s="34" t="n">
         <v>4</v>
       </c>
-      <c r="E29" s="28" t="n">
+      <c r="E29" s="44" t="n">
         <f aca="false">P_dmp</f>
-        <v>0.01</v>
+        <v>0.004</v>
       </c>
       <c r="F29" s="28" t="n">
         <f aca="false">D29*E29</f>
-        <v>0.04</v>
+        <v>0.016</v>
       </c>
       <c r="G29" s="34" t="n">
         <v>230</v>
@@ -7198,7 +7316,7 @@
       </c>
       <c r="I29" s="12" t="n">
         <f aca="false">F29*1000/(G29*H29)</f>
-        <v>0.183066361556064</v>
+        <v>0.0732265446224256</v>
       </c>
       <c r="J29" s="34" t="n">
         <f aca="false">INDEX({6,10,16,20,25,32,40,50,63,80,100,125,160,200,250},MATCH(TRUE(),INDEX({6,10,16,20,25,32,40,50,63,80,100,125,160,200,250}&gt;=I29*k_sig,0),0))</f>
@@ -7207,22 +7325,24 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="16" t="s">
-        <v>360</v>
-      </c>
-      <c r="B30" s="16"/>
+        <v>377</v>
+      </c>
+      <c r="B30" s="16" t="s">
+        <v>378</v>
+      </c>
       <c r="C30" s="4" t="s">
-        <v>341</v>
+        <v>347</v>
       </c>
       <c r="D30" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="E30" s="28" t="n">
+      <c r="E30" s="44" t="n">
         <f aca="false">P_ddc</f>
-        <v>0.3</v>
+        <v>0.15</v>
       </c>
       <c r="F30" s="28" t="n">
         <f aca="false">D30*E30</f>
-        <v>0.3</v>
+        <v>0.15</v>
       </c>
       <c r="G30" s="34" t="n">
         <v>230</v>
@@ -7233,7 +7353,7 @@
       </c>
       <c r="I30" s="12" t="n">
         <f aca="false">F30*1000/(G30*H30)</f>
-        <v>1.37299771167048</v>
+        <v>0.68649885583524</v>
       </c>
       <c r="J30" s="34" t="n">
         <f aca="false">INDEX({6,10,16,20,25,32,40,50,63,80,100,125,160,200,250},MATCH(TRUE(),INDEX({6,10,16,20,25,32,40,50,63,80,100,125,160,200,250}&gt;=I30*k_sig,0),0))</f>
@@ -7245,21 +7365,21 @@
         <v>11</v>
       </c>
       <c r="B31" s="41" t="s">
-        <v>361</v>
+        <v>379</v>
       </c>
       <c r="C31" s="23" t="s">
-        <v>343</v>
+        <v>349</v>
       </c>
       <c r="D31" s="36" t="n">
         <v>1</v>
       </c>
-      <c r="E31" s="38" t="n">
+      <c r="E31" s="42" t="n">
         <f aca="false">ROUND(MAX('KS HESABI'!F51/EER,'KS HESABI'!F52*dus/COP),1)</f>
-        <v>50</v>
+        <v>53.6</v>
       </c>
       <c r="F31" s="38" t="n">
         <f aca="false">D31*E31</f>
-        <v>50</v>
+        <v>53.6</v>
       </c>
       <c r="G31" s="36" t="n">
         <f aca="false">U_v</f>
@@ -7269,13 +7389,13 @@
         <f aca="false">cos_du</f>
         <v>0.92</v>
       </c>
-      <c r="I31" s="42" t="n">
+      <c r="I31" s="43" t="n">
         <f aca="false">F31*1000/(SQRT(3)*G31*H31)</f>
-        <v>78.4443300529383</v>
+        <v>84.0923218167498</v>
       </c>
       <c r="J31" s="36" t="n">
         <f aca="false">INDEX({6,10,16,20,25,32,40,50,63,80,100,125,160,200,250},MATCH(TRUE(),INDEX({6,10,16,20,25,32,40,50,63,80,100,125,160,200,250}&gt;=I31*k_sig,0),0))</f>
-        <v>100</v>
+        <v>125</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7283,21 +7403,21 @@
         <v>12</v>
       </c>
       <c r="B32" s="41" t="s">
-        <v>362</v>
+        <v>380</v>
       </c>
       <c r="C32" s="23" t="s">
-        <v>343</v>
+        <v>349</v>
       </c>
       <c r="D32" s="36" t="n">
         <v>1</v>
       </c>
-      <c r="E32" s="38" t="n">
+      <c r="E32" s="42" t="n">
         <f aca="false">ROUND(MAX('KS HESABI'!F51/EER,'KS HESABI'!F52*dus/COP),1)</f>
-        <v>50</v>
+        <v>53.6</v>
       </c>
       <c r="F32" s="38" t="n">
         <f aca="false">D32*E32</f>
-        <v>50</v>
+        <v>53.6</v>
       </c>
       <c r="G32" s="36" t="n">
         <f aca="false">U_v</f>
@@ -7307,38 +7427,38 @@
         <f aca="false">cos_du</f>
         <v>0.92</v>
       </c>
-      <c r="I32" s="42" t="n">
+      <c r="I32" s="43" t="n">
         <f aca="false">F32*1000/(SQRT(3)*G32*H32)</f>
-        <v>78.4443300529383</v>
+        <v>84.0923218167498</v>
       </c>
       <c r="J32" s="36" t="n">
         <f aca="false">INDEX({6,10,16,20,25,32,40,50,63,80,100,125,160,200,250},MATCH(TRUE(),INDEX({6,10,16,20,25,32,40,50,63,80,100,125,160,200,250}&gt;=I32*k_sig,0),0))</f>
-        <v>100</v>
+        <v>125</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="24"/>
       <c r="B33" s="24"/>
       <c r="C33" s="23" t="s">
-        <v>363</v>
+        <v>381</v>
       </c>
       <c r="D33" s="24"/>
       <c r="E33" s="24"/>
       <c r="F33" s="31" t="n">
         <f aca="false">F5+F10+F11+F12+F17+F18+F19+F24+F25+F26+F31+F32</f>
-        <v>540.16</v>
+        <v>549.064</v>
       </c>
       <c r="G33" s="24"/>
       <c r="H33" s="24"/>
       <c r="I33" s="31" t="n">
         <f aca="false">I5+I10+I11+I12+I17+I18+I19+I24+I25+I26+I31+I32</f>
-        <v>839.851751191954</v>
+        <v>854.747388137047</v>
       </c>
       <c r="J33" s="24"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C35" s="2" t="s">
-        <v>364</v>
+        <v>382</v>
       </c>
     </row>
   </sheetData>
@@ -7367,125 +7487,125 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>365</v>
+        <v>383</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
-        <v>366</v>
+        <v>384</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>367</v>
+        <v>385</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>368</v>
+        <v>386</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>369</v>
+        <v>387</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>370</v>
-      </c>
-      <c r="B4" s="43" t="n">
+        <v>388</v>
+      </c>
+      <c r="B4" s="45" t="n">
         <f aca="false">VLOOKUP("MARKET",TIP_TABLO,4,FALSE())</f>
         <v>0.15</v>
       </c>
       <c r="C4" s="16" t="s">
-        <v>371</v>
+        <v>389</v>
       </c>
       <c r="D4" s="12" t="n">
         <f aca="false">B4*130</f>
         <v>19.5</v>
       </c>
       <c r="E4" s="13" t="s">
-        <v>372</v>
+        <v>390</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>373</v>
+        <v>391</v>
       </c>
       <c r="B5" s="11" t="n">
         <v>12</v>
       </c>
       <c r="C5" s="16" t="s">
-        <v>368</v>
+        <v>386</v>
       </c>
       <c r="D5" s="12" t="n">
         <f aca="false">B5</f>
         <v>12</v>
       </c>
       <c r="E5" s="13" t="s">
-        <v>374</v>
+        <v>392</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>375</v>
+        <v>393</v>
       </c>
       <c r="B6" s="11" t="n">
         <v>10</v>
       </c>
       <c r="C6" s="16" t="s">
-        <v>368</v>
+        <v>386</v>
       </c>
       <c r="D6" s="12" t="n">
         <f aca="false">B6</f>
         <v>10</v>
       </c>
       <c r="E6" s="13" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>376</v>
-      </c>
-      <c r="B7" s="43" t="n">
+        <v>394</v>
+      </c>
+      <c r="B7" s="45" t="n">
         <f aca="false">U_cati</f>
         <v>0.2</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D7" s="12" t="n">
         <f aca="false">B7*25</f>
         <v>5</v>
       </c>
       <c r="E7" s="13" t="s">
-        <v>377</v>
+        <v>395</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>378</v>
+        <v>396</v>
       </c>
       <c r="B8" s="11" t="n">
         <v>8</v>
       </c>
       <c r="C8" s="16" t="s">
-        <v>368</v>
+        <v>386</v>
       </c>
       <c r="D8" s="12" t="n">
         <f aca="false">B8</f>
         <v>8</v>
       </c>
       <c r="E8" s="13" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="9" t="s">
-        <v>379</v>
+        <v>397</v>
       </c>
       <c r="B9" s="4"/>
       <c r="C9" s="16"/>
-      <c r="D9" s="44" t="n">
+      <c r="D9" s="46" t="n">
         <f aca="false">SUM(D4:D8)</f>
         <v>54.5</v>
       </c>
@@ -7493,7 +7613,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>380</v>
+        <v>398</v>
       </c>
       <c r="B10" s="4"/>
       <c r="C10" s="16"/>
@@ -7502,12 +7622,12 @@
         <v>72</v>
       </c>
       <c r="E10" s="13" t="s">
-        <v>381</v>
+        <v>399</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>382</v>
+        <v>400</v>
       </c>
       <c r="B11" s="4"/>
       <c r="C11" s="16"/>
@@ -7516,7 +7636,7 @@
         <v>1.32110091743119</v>
       </c>
       <c r="E11" s="13" t="s">
-        <v>383</v>
+        <v>401</v>
       </c>
     </row>
   </sheetData>

</xml_diff>